<commit_message>
Added Business Rule Exception
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harih\OneDrive\Documents\UiPath\Adjustments\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{431CD5F4-2BD5-46B6-BBFA-8BCF0C6B8662}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EC10D1C-147A-44BD-B026-29CE5DC35AE3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="19200" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="357">
   <si>
     <t>Name</t>
   </si>
@@ -1093,6 +1093,9 @@
   </si>
   <si>
     <t>Entered Transaction Number is Invalid</t>
+  </si>
+  <si>
+    <t>BRE_DuplicateAdjustmentNumber</t>
   </si>
 </sst>
 </file>
@@ -1485,7 +1488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1050"/>
+  <dimension ref="A1:Z1053"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="49.54296875" customWidth="1"/>
@@ -2651,99 +2654,94 @@
         <v>355</v>
       </c>
     </row>
-    <row r="156" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="157" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A157" t="s">
-        <v>301</v>
-      </c>
-      <c r="B157">
-        <v>5</v>
-      </c>
-      <c r="C157" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A158" t="s">
-        <v>351</v>
-      </c>
-      <c r="B158">
-        <v>5</v>
-      </c>
-      <c r="C158" t="s">
-        <v>48</v>
-      </c>
-    </row>
+    <row r="156" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A156" t="s">
+        <v>356</v>
+      </c>
+      <c r="B156" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="158" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="159" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="160" spans="1:3" ht="14.25" customHeight="1">
       <c r="A160" t="s">
+        <v>301</v>
+      </c>
+      <c r="B160">
+        <v>5</v>
+      </c>
+      <c r="C160" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A161" t="s">
+        <v>351</v>
+      </c>
+      <c r="B161">
+        <v>5</v>
+      </c>
+      <c r="C161" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="163" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A163" t="s">
         <v>348</v>
       </c>
-      <c r="B160" t="s">
+      <c r="B163" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="161" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A161" t="s">
+    <row r="164" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A164" t="s">
         <v>352</v>
       </c>
-      <c r="B161" t="s">
+      <c r="B164" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="162" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="163" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="164" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="165" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="166" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="167" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="168" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="169" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="170" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="171" spans="1:2" s="6" customFormat="1" ht="14.5"/>
-    <row r="172" spans="1:2" s="6" customFormat="1" ht="14.5">
-      <c r="B172" s="7"/>
-    </row>
-    <row r="173" spans="1:2" s="6" customFormat="1" ht="14.5">
-      <c r="B173" s="7"/>
-    </row>
-    <row r="174" spans="1:2" s="6" customFormat="1" ht="14.5">
-      <c r="B174" s="7"/>
-    </row>
-    <row r="175" spans="1:2" s="6" customFormat="1" ht="14.5"/>
-    <row r="176" spans="1:2" s="6" customFormat="1" ht="14.5">
+    <row r="165" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="166" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="167" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="168" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="169" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="170" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="171" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="172" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="173" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="174" spans="1:3" s="6" customFormat="1" ht="14.5"/>
+    <row r="175" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B175" s="7"/>
+    </row>
+    <row r="176" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="B176" s="7"/>
     </row>
     <row r="177" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="B177" s="7"/>
     </row>
-    <row r="178" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B178" s="7"/>
-    </row>
-    <row r="179" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="180" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A180" s="6"/>
+    <row r="178" spans="1:3" s="6" customFormat="1" ht="14.5"/>
+    <row r="179" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B179" s="7"/>
+    </row>
+    <row r="180" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="B180" s="7"/>
-      <c r="C180" s="6"/>
-    </row>
-    <row r="181" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A181" s="6"/>
-      <c r="B181" s="8"/>
-      <c r="C181" s="6"/>
-    </row>
-    <row r="182" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A182" s="6"/>
-      <c r="B182" s="7"/>
-      <c r="C182" s="6"/>
-    </row>
+    </row>
+    <row r="181" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B181" s="7"/>
+    </row>
+    <row r="182" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="183" spans="1:3" ht="14.25" customHeight="1">
       <c r="A183" s="6"/>
-      <c r="B183" s="6"/>
+      <c r="B183" s="7"/>
       <c r="C183" s="6"/>
     </row>
     <row r="184" spans="1:3" ht="14.25" customHeight="1">
       <c r="A184" s="6"/>
-      <c r="B184" s="5"/>
+      <c r="B184" s="8"/>
       <c r="C184" s="6"/>
     </row>
     <row r="185" spans="1:3" ht="14.25" customHeight="1">
@@ -2753,12 +2751,12 @@
     </row>
     <row r="186" spans="1:3" ht="14.25" customHeight="1">
       <c r="A186" s="6"/>
-      <c r="B186" s="8"/>
+      <c r="B186" s="6"/>
       <c r="C186" s="6"/>
     </row>
     <row r="187" spans="1:3" ht="14.25" customHeight="1">
       <c r="A187" s="6"/>
-      <c r="B187" s="6"/>
+      <c r="B187" s="5"/>
       <c r="C187" s="6"/>
     </row>
     <row r="188" spans="1:3" ht="14.25" customHeight="1">
@@ -2766,34 +2764,46 @@
       <c r="B188" s="7"/>
       <c r="C188" s="6"/>
     </row>
-    <row r="189" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="189" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A189" s="6"/>
+      <c r="B189" s="8"/>
+      <c r="C189" s="6"/>
+    </row>
     <row r="190" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B190" s="5"/>
+      <c r="A190" s="6"/>
+      <c r="B190" s="6"/>
+      <c r="C190" s="6"/>
     </row>
     <row r="191" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A191" s="6"/>
       <c r="B191" s="7"/>
-    </row>
-    <row r="192" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B192" s="8"/>
-    </row>
-    <row r="193" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="194" spans="1:1" ht="14.25" customHeight="1">
-      <c r="A194" s="6"/>
-    </row>
-    <row r="195" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="196" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="197" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="198" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="199" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="200" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="201" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="202" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="203" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="204" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="205" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="206" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="207" spans="1:1" ht="14.25" customHeight="1"/>
-    <row r="208" spans="1:1" ht="14.25" customHeight="1"/>
+      <c r="C191" s="6"/>
+    </row>
+    <row r="192" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="193" spans="1:2" ht="14.25" customHeight="1">
+      <c r="B193" s="5"/>
+    </row>
+    <row r="194" spans="1:2" ht="14.25" customHeight="1">
+      <c r="B194" s="7"/>
+    </row>
+    <row r="195" spans="1:2" ht="14.25" customHeight="1">
+      <c r="B195" s="8"/>
+    </row>
+    <row r="196" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="197" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A197" s="6"/>
+    </row>
+    <row r="198" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="199" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="200" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="201" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="202" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="203" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="204" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="205" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="206" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="207" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="208" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="209" ht="14.25" customHeight="1"/>
     <row r="210" ht="14.25" customHeight="1"/>
     <row r="211" ht="14.25" customHeight="1"/>
@@ -3636,6 +3646,9 @@
     <row r="1048" ht="14.25" customHeight="1"/>
     <row r="1049" ht="14.25" customHeight="1"/>
     <row r="1050" ht="14.25" customHeight="1"/>
+    <row r="1051" ht="14.25" customHeight="1"/>
+    <row r="1052" ht="14.25" customHeight="1"/>
+    <row r="1053" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated Config file and Log messages
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,22 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harih\OneDrive\Documents\UiPath\Adjustments\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EC10D1C-147A-44BD-B026-29CE5DC35AE3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C16995FB-7C24-4456-A580-A8AFC314F030}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="19200" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
     <sheet name="Constants" sheetId="2" r:id="rId2"/>
     <sheet name="Assets" sheetId="3" r:id="rId3"/>
-    <sheet name="TCP DEL" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="266">
   <si>
     <t>Name</t>
   </si>
@@ -410,9 +409,6 @@
     <t>TimeStamp</t>
   </si>
   <si>
-    <t>Log_ValidationStatus</t>
-  </si>
-  <si>
     <t>BotStatus_BRE</t>
   </si>
   <si>
@@ -483,9 +479,6 @@
     <t>TimeOut_Logout</t>
   </si>
   <si>
-    <t>Treasury Confirmation Process - User Input Form</t>
-  </si>
-  <si>
     <t>ColName_Status</t>
   </si>
   <si>
@@ -501,345 +494,27 @@
     <t>Validating Input file for invalid data</t>
   </si>
   <si>
-    <t>Accomplished Date</t>
-  </si>
-  <si>
-    <t>ColName_AccomplishedDate</t>
-  </si>
-  <si>
-    <t>Payment Instruction</t>
-  </si>
-  <si>
-    <t>ColName_PaymentInstruction</t>
-  </si>
-  <si>
-    <t>Accomplished Date - Invalid Date Format</t>
-  </si>
-  <si>
-    <t>BotStatus_AccomplishedDate_InvalidDateFormat</t>
-  </si>
-  <si>
-    <t>BotStatus_PaymentInstruction_InvalidData</t>
-  </si>
-  <si>
-    <t>PaymentInstruction - Invalid Data</t>
-  </si>
-  <si>
-    <t>Range Sequence</t>
-  </si>
-  <si>
-    <t>From</t>
-  </si>
-  <si>
-    <t>To</t>
-  </si>
-  <si>
-    <t>ColName_RangeSequence</t>
-  </si>
-  <si>
-    <t>ColName_From</t>
-  </si>
-  <si>
-    <t>ColName_To</t>
-  </si>
-  <si>
-    <t>BotStatus_RangeSequence_InvalidData</t>
-  </si>
-  <si>
-    <t>BotStatus_From_InvalidData</t>
-  </si>
-  <si>
-    <t>BotStatus_To_InvalidData</t>
-  </si>
-  <si>
-    <t>RangeSequence - Invalid Data</t>
-  </si>
-  <si>
-    <t>From - Invalid Data</t>
-  </si>
-  <si>
-    <t>To - Invalid Data</t>
-  </si>
-  <si>
-    <t>Log_GetUniquePaymentInstructions</t>
-  </si>
-  <si>
-    <t>Getting Unique Payment Instructions from valid data</t>
-  </si>
-  <si>
     <t>Log_ValidateInputFileSuccess</t>
   </si>
   <si>
     <t>Validating Input file for invalid data - Success</t>
   </si>
   <si>
-    <t>Log_GetUniquePaymentInstructionsSuccess</t>
-  </si>
-  <si>
-    <t>Getting Unique Payment Instructions from valid data - Success</t>
-  </si>
-  <si>
-    <t>Log_UniquePaymentInstructionsCount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of Unique Payment Instructions - </t>
-  </si>
-  <si>
     <t>SE_ErrMsg_MaxRetry</t>
   </si>
   <si>
-    <t>DOL Federal Administrator</t>
-  </si>
-  <si>
-    <t>Log_NavigateToTreasuryConfirmation</t>
-  </si>
-  <si>
-    <t>Navigating to Treasury Confirmation</t>
-  </si>
-  <si>
-    <t>Log_NavigateToTreasuryConfirmationSuccess</t>
-  </si>
-  <si>
-    <t>Navigating to Treasury Confirmation - Success</t>
-  </si>
-  <si>
-    <t>SE_ErrMsg_FederalAdministratorNotDisplayed</t>
-  </si>
-  <si>
-    <t>DOL Federal Administrator Not Displayed</t>
-  </si>
-  <si>
-    <t>SE_ErrMsg_TreasuryConfirmationNotDisplayed</t>
-  </si>
-  <si>
-    <t>Treasury Confirmation Not Displayed</t>
-  </si>
-  <si>
-    <t>ColName_ProcessType</t>
-  </si>
-  <si>
-    <t>ProcessType</t>
-  </si>
-  <si>
-    <t>Transaction Complete</t>
-  </si>
-  <si>
-    <t>ColName_RequestNumber</t>
-  </si>
-  <si>
-    <t>Request Number</t>
-  </si>
-  <si>
-    <t>ColName_ReferenceAssignedbyAdmin</t>
-  </si>
-  <si>
-    <t>Reference Assigned by Admin</t>
-  </si>
-  <si>
-    <t>Date Sent to Treasury</t>
-  </si>
-  <si>
-    <t>ColName_DateSentToTreasury</t>
-  </si>
-  <si>
-    <t>BotStatus_DateSentToTreasury_InvalidDateFormat</t>
-  </si>
-  <si>
-    <t>Date Sent To Treasury - Invalid Date Format</t>
-  </si>
-  <si>
-    <t>Treasury Confirmation - Report</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Attached is the bot generated Treasury Confirmation Report. </t>
-  </si>
-  <si>
-    <t>Treasury Confirmation - Error Occurred</t>
-  </si>
-  <si>
-    <t>MaxNumOfValidationLoops</t>
-  </si>
-  <si>
-    <t>Number</t>
-  </si>
-  <si>
     <t>Status_InProgress</t>
   </si>
   <si>
     <t>In Progress - Check Concurrent Manager</t>
   </si>
   <si>
-    <t>Confirm</t>
-  </si>
-  <si>
-    <t>BackOut</t>
-  </si>
-  <si>
-    <t>ProcessType_Confirm</t>
-  </si>
-  <si>
-    <t>ProcessType_BackOut</t>
-  </si>
-  <si>
-    <t>BRE_InvalidPaymentInstructon</t>
-  </si>
-  <si>
-    <t>Entered 'PaymentInstruction' is invalid</t>
-  </si>
-  <si>
-    <t>Log_PaymentCount</t>
-  </si>
-  <si>
-    <t>Account Entries need to be created</t>
-  </si>
-  <si>
-    <t>BRE_AccountEntryError</t>
-  </si>
-  <si>
-    <t>Log_RequestNumber</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Request Number - </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Payment Count - </t>
-  </si>
-  <si>
-    <t>Log_Status</t>
-  </si>
-  <si>
-    <t>Status after Validation -</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Intitial Status - </t>
-  </si>
-  <si>
-    <t>Log_LogErrorMessage</t>
-  </si>
-  <si>
-    <t>Log_ConfirmationEntry</t>
-  </si>
-  <si>
-    <t>Log_ConfirmationEntrySuccess</t>
-  </si>
-  <si>
-    <t>Entering Confirmation Process</t>
-  </si>
-  <si>
-    <t>Entering MultipleRange Type</t>
-  </si>
-  <si>
-    <t>Log_MultipleRangeEntry</t>
-  </si>
-  <si>
-    <t>Log_MultipleRangeEntrySuccess</t>
-  </si>
-  <si>
-    <t>Log_SingleRangeEntry</t>
-  </si>
-  <si>
-    <t>Entering SingleRange Type</t>
-  </si>
-  <si>
     <t>Handling security warnings - Success</t>
   </si>
   <si>
-    <t>Confirmation Process - Success</t>
-  </si>
-  <si>
-    <t>MultipleRange Type - Success</t>
-  </si>
-  <si>
-    <t>Log_BackOutEntry</t>
-  </si>
-  <si>
-    <t>Entering BackOut Process</t>
-  </si>
-  <si>
-    <t>Log_BackOutEntrySuccess</t>
-  </si>
-  <si>
-    <t>BackOut Process - Success</t>
-  </si>
-  <si>
-    <t>SingleRange Type - Success</t>
-  </si>
-  <si>
-    <t>Validating Payment Instruction</t>
-  </si>
-  <si>
-    <t>Log_ValidationPaymentInstruction</t>
-  </si>
-  <si>
-    <t>Log_ValidationPaymentInstructionSuccess</t>
-  </si>
-  <si>
-    <t>Validating Payment Instruction - Success</t>
-  </si>
-  <si>
-    <t>Log_ViewLogsEntry</t>
-  </si>
-  <si>
-    <t>Log_ViewLogsEntrySuccess</t>
-  </si>
-  <si>
-    <t>Log_SingleRangeEntrySuccess</t>
-  </si>
-  <si>
-    <t>Log_ReOpenTreasuryConfirmation</t>
-  </si>
-  <si>
-    <t>ReOpening Treasury Confirmation</t>
-  </si>
-  <si>
-    <t>Log_ReOpenTreasuryConfirmationSuccess</t>
-  </si>
-  <si>
-    <t>ReOpening Treasury Confirmation - Success</t>
-  </si>
-  <si>
-    <t>BRE_FieldsNotMatch</t>
-  </si>
-  <si>
-    <t>BRE_InvalidBackOut</t>
-  </si>
-  <si>
-    <t>Invalid Back Out</t>
-  </si>
-  <si>
-    <t>Payment Instruction Fields did not match</t>
-  </si>
-  <si>
-    <t>TimeOut_BackOutRequestNumberNote</t>
-  </si>
-  <si>
-    <t>ViewLog_StartIndex</t>
-  </si>
-  <si>
-    <t>ViewLog_EndIndex</t>
-  </si>
-  <si>
-    <t>Start of log messages from FND_FILE</t>
-  </si>
-  <si>
-    <t>End of log messages from FND_FILE</t>
-  </si>
-  <si>
-    <t>Log Message(s) for Unconfirmed Payment Instruction -</t>
-  </si>
-  <si>
-    <t>Extracting Log Message(s) for Unconfirmed Payment Instruction</t>
-  </si>
-  <si>
-    <t>Extracting Log Message(s) for Unconfirmed Payment Instruction - Success</t>
-  </si>
-  <si>
     <t>TimeOut_ErrorDisplayed</t>
   </si>
   <si>
-    <t>TimeOut_PaymentInstructionDropdownDisplayed</t>
-  </si>
-  <si>
     <t>Status_Confirmed</t>
   </si>
   <si>
@@ -852,15 +527,6 @@
     <t>Unconfirmed</t>
   </si>
   <si>
-    <t>AdjustRowHeight</t>
-  </si>
-  <si>
-    <t>in number</t>
-  </si>
-  <si>
-    <t>gmahesh2789@gmail.com; hariharangouri@gmail.com</t>
-  </si>
-  <si>
     <t>gmahesh2789@gmail.com; hariharangouri@gmail.com; sunil.melam@gmail.com</t>
   </si>
   <si>
@@ -1083,12 +749,6 @@
     <t>TimeOut_TimeOut_AcitivityNamesDisplayed</t>
   </si>
   <si>
-    <t>Field_WrongValue</t>
-  </si>
-  <si>
-    <t>Entered value is wrong</t>
-  </si>
-  <si>
     <t>BRE_InvalidTransactionNumber</t>
   </si>
   <si>
@@ -1096,6 +756,72 @@
   </si>
   <si>
     <t>BRE_DuplicateAdjustmentNumber</t>
+  </si>
+  <si>
+    <t>TimeOut_IEModeEdgeBrowser</t>
+  </si>
+  <si>
+    <t>Log_EmptyCommentsTabField</t>
+  </si>
+  <si>
+    <t>Comment Tab fields are empty</t>
+  </si>
+  <si>
+    <t>Log_AdjustmentNumberExtract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extracted Adjustment Number is - </t>
+  </si>
+  <si>
+    <t>Log_NavigatingToAdjustStart</t>
+  </si>
+  <si>
+    <t>Navigating to Adjustments Started</t>
+  </si>
+  <si>
+    <t>Log_NavigatingToAdjustSuccess</t>
+  </si>
+  <si>
+    <t>Navigating to Adjustments Success</t>
+  </si>
+  <si>
+    <t>Adjusting Transaction Amount started</t>
+  </si>
+  <si>
+    <t>Log_AdjustmentStart</t>
+  </si>
+  <si>
+    <t>Log_AdjustmentSuccess</t>
+  </si>
+  <si>
+    <t>Adjusting Transaction Amount success</t>
+  </si>
+  <si>
+    <t>TimeOut_AdjustmentReasonsPanelDisplayed</t>
+  </si>
+  <si>
+    <t>BRE_ReasonError</t>
+  </si>
+  <si>
+    <t>Entered Reason field is incorrect</t>
+  </si>
+  <si>
+    <t>TimeOut_StatusPanelDisplayed</t>
+  </si>
+  <si>
+    <t>BRE_StatusError</t>
+  </si>
+  <si>
+    <t>Entered Status field is incorrect</t>
+  </si>
+  <si>
+    <t>TimeOut_AdjustmentInformationDisplayed</t>
+  </si>
+  <si>
+    <t>BRE_ActivityNamesError</t>
+  </si>
+  <si>
+    <t>Entered Activity Name Field is incorrect</t>
   </si>
 </sst>
 </file>
@@ -1148,7 +874,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -1171,7 +897,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
@@ -1488,7 +1213,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1053"/>
+  <dimension ref="A1:Z1068"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="49.54296875" customWidth="1"/>
@@ -1541,7 +1266,7 @@
         <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>330</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -1591,7 +1316,7 @@
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>42</v>
@@ -1603,10 +1328,10 @@
     </row>
     <row r="12" spans="1:26" ht="15" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>327</v>
+        <v>216</v>
       </c>
       <c r="B12" t="s">
-        <v>328</v>
+        <v>217</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="15" customHeight="1">
@@ -1637,74 +1362,74 @@
     </row>
     <row r="16" spans="1:26" ht="14.5">
       <c r="A16" s="2" t="s">
-        <v>309</v>
+        <v>198</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>306</v>
+        <v>195</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="15" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>322</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>320</v>
+        <v>211</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>302</v>
+        <v>193</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="15" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>305</v>
+        <v>196</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="15" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>303</v>
+        <v>197</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>323</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>321</v>
+        <v>212</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>314</v>
+        <v>204</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>313</v>
+        <v>201</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.5">
       <c r="A24" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>154</v>
+        <v>151</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="15.5" customHeight="1">
@@ -1717,36 +1442,36 @@
     </row>
     <row r="27" spans="1:2" ht="14.5">
       <c r="A27" t="s">
-        <v>331</v>
+        <v>220</v>
       </c>
       <c r="B27" t="s">
-        <v>334</v>
+        <v>223</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.5">
       <c r="A28" t="s">
-        <v>332</v>
+        <v>221</v>
       </c>
       <c r="B28" t="s">
-        <v>333</v>
+        <v>222</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="15" customHeight="1">
       <c r="A29" t="s">
-        <v>319</v>
+        <v>208</v>
       </c>
       <c r="B29" t="s">
-        <v>318</v>
+        <v>207</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="12.5" customHeight="1"/>
     <row r="31" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="32" spans="1:2" ht="14.25" customHeight="1">
       <c r="A32" t="s">
+        <v>128</v>
+      </c>
+      <c r="B32" t="s">
         <v>129</v>
-      </c>
-      <c r="B32" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1">
@@ -1754,7 +1479,7 @@
         <v>67</v>
       </c>
       <c r="B33" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1"/>
@@ -1763,7 +1488,7 @@
         <v>49</v>
       </c>
       <c r="B35" t="s">
-        <v>316</v>
+        <v>205</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1">
@@ -1771,13 +1496,13 @@
         <v>66</v>
       </c>
       <c r="B36" t="s">
-        <v>329</v>
+        <v>218</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>317</v>
+        <v>206</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="15" customHeight="1">
@@ -1793,7 +1518,7 @@
         <v>64</v>
       </c>
       <c r="B41" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="15" customHeight="1">
@@ -1814,50 +1539,50 @@
     </row>
     <row r="45" spans="1:2" ht="14.5">
       <c r="A45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B45" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.5">
       <c r="A46" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="B46" t="s">
-        <v>181</v>
+        <v>157</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.5">
       <c r="A47" t="s">
-        <v>336</v>
+        <v>225</v>
       </c>
       <c r="B47" t="s">
-        <v>335</v>
+        <v>224</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.5">
       <c r="A48" t="s">
-        <v>342</v>
+        <v>231</v>
       </c>
       <c r="B48" t="s">
-        <v>341</v>
+        <v>230</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.5">
       <c r="A49" t="s">
+        <v>144</v>
+      </c>
+      <c r="B49" t="s">
         <v>145</v>
-      </c>
-      <c r="B49" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.5">
       <c r="A50" t="s">
+        <v>146</v>
+      </c>
+      <c r="B50" t="s">
         <v>147</v>
-      </c>
-      <c r="B50" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="14.5">
@@ -1870,26 +1595,26 @@
     </row>
     <row r="52" spans="1:2" ht="14.5">
       <c r="A52" t="s">
+        <v>148</v>
+      </c>
+      <c r="B52" t="s">
         <v>149</v>
-      </c>
-      <c r="B52" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="53" spans="1:2" s="9" customFormat="1" ht="14.5">
       <c r="A53" s="9" t="s">
-        <v>279</v>
+        <v>168</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>281</v>
+        <v>170</v>
       </c>
     </row>
     <row r="54" spans="1:2" s="9" customFormat="1" ht="14.5">
       <c r="A54" s="9" t="s">
-        <v>280</v>
+        <v>169</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>282</v>
+        <v>171</v>
       </c>
     </row>
     <row r="55" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
@@ -1905,413 +1630,402 @@
         <v>124</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>238</v>
+        <v>161</v>
       </c>
     </row>
     <row r="57" spans="1:2" s="9" customFormat="1" ht="14.5">
-      <c r="A57" s="14" t="s">
-        <v>337</v>
-      </c>
-      <c r="B57" s="14" t="s">
-        <v>338</v>
+      <c r="A57" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="B57" s="13" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="58" spans="1:2" s="9" customFormat="1" ht="14.5">
-      <c r="A58" s="14" t="s">
-        <v>339</v>
-      </c>
-      <c r="B58" s="14" t="s">
-        <v>340</v>
+      <c r="A58" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="B58" s="13" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="59" spans="1:2" s="9" customFormat="1" ht="14.5">
-      <c r="A59" s="14" t="s">
-        <v>285</v>
-      </c>
-      <c r="B59" s="14" t="s">
-        <v>287</v>
+      <c r="A59" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="B59" s="13" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="60" spans="1:2" s="9" customFormat="1" ht="14.5">
-      <c r="A60" s="14" t="s">
-        <v>286</v>
-      </c>
-      <c r="B60" s="14" t="s">
-        <v>288</v>
+      <c r="A60" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="B60" s="13" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="14.25" customHeight="1">
       <c r="A61" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="B61" t="s">
         <v>143</v>
       </c>
-      <c r="B61" t="s">
-        <v>144</v>
-      </c>
     </row>
     <row r="62" spans="1:2" s="9" customFormat="1" ht="14.5">
-      <c r="A62" s="14"/>
-      <c r="B62" s="14"/>
-    </row>
-    <row r="63" spans="1:2" ht="14.5">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2"/>
-    </row>
-    <row r="64" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A62" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="B62" s="13" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" s="9" customFormat="1" ht="14.5">
+      <c r="A63" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="B63" s="13" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" s="9" customFormat="1" ht="14.5">
       <c r="A64" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="B64" s="9" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" ht="15" customHeight="1">
-      <c r="A65" t="s">
-        <v>95</v>
-      </c>
-      <c r="B65" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
+        <v>249</v>
+      </c>
+      <c r="B64" s="13" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" s="9" customFormat="1" ht="14.5">
+      <c r="A65" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="B65" s="13" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" s="9" customFormat="1" ht="14.5">
       <c r="A66" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="B66" s="9" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
+        <v>254</v>
+      </c>
+      <c r="B66" s="13" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" s="9" customFormat="1" ht="14.5">
       <c r="A67" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="B67" s="9" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A68" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B68" s="9" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A69" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="B69" s="14" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A70" s="9" t="s">
-        <v>283</v>
-      </c>
-      <c r="B70" s="9" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A71" s="9" t="s">
-        <v>344</v>
-      </c>
-      <c r="B71" s="9" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" ht="14.25" customHeight="1">
+        <v>255</v>
+      </c>
+      <c r="B67" s="13" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" s="9" customFormat="1" ht="14.5">
+      <c r="B68" s="13"/>
+    </row>
+    <row r="69" spans="1:2" s="9" customFormat="1" ht="14.5">
+      <c r="B69" s="13"/>
+    </row>
+    <row r="70" spans="1:2" s="9" customFormat="1" ht="14.5">
+      <c r="B70" s="13"/>
+    </row>
+    <row r="71" spans="1:2" s="9" customFormat="1" ht="14.5">
+      <c r="B71" s="13"/>
+    </row>
+    <row r="72" spans="1:2" ht="14.5">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
     </row>
-    <row r="73" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A73" s="6" t="s">
+    <row r="73" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A73" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B73" s="9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" ht="15" customHeight="1">
+      <c r="A74" t="s">
+        <v>95</v>
+      </c>
+      <c r="B74" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A75" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B75" s="9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A76" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B76" s="9" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A77" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B77" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A78" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="B78" s="13" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A79" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="B79" s="9" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A80" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="B80" s="9" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A81" s="2"/>
+      <c r="B81" s="2"/>
+    </row>
+    <row r="82" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A82" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B73" s="7">
+      <c r="B82" s="7">
         <v>2000</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C82" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A74" s="6" t="s">
+    <row r="83" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A83" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B74">
+      <c r="B83">
         <v>1</v>
       </c>
-      <c r="C74" t="s">
+      <c r="C83" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A75" s="6" t="s">
+    <row r="84" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A84" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B75" s="7" t="s">
+      <c r="B84" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="C75" s="6"/>
-    </row>
-    <row r="76" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A76" s="6" t="s">
+      <c r="C84" s="6"/>
+    </row>
+    <row r="85" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A85" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B76" s="7">
+      <c r="B85" s="7">
         <v>3</v>
       </c>
-      <c r="C76" s="6"/>
-    </row>
-    <row r="77" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A77" s="6" t="s">
+      <c r="C85" s="6"/>
+    </row>
+    <row r="86" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A86" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B77" s="7">
+      <c r="B86" s="7">
         <v>3</v>
       </c>
-      <c r="C77" t="s">
+      <c r="C86" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="14.5"/>
-    <row r="79" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A79" t="s">
+    <row r="87" spans="1:3" ht="14.5"/>
+    <row r="88" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A88" t="s">
         <v>91</v>
       </c>
-      <c r="B79" s="5" t="s">
+      <c r="B88" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="81" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A81" t="s">
-        <v>109</v>
-      </c>
-      <c r="B81" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A82" t="s">
-        <v>97</v>
-      </c>
-      <c r="B82" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="84" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A84" t="s">
-        <v>111</v>
-      </c>
-      <c r="B84" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A85" t="s">
-        <v>117</v>
-      </c>
-      <c r="B85" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A86" t="s">
-        <v>112</v>
-      </c>
-      <c r="B86" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A87" t="s">
-        <v>118</v>
-      </c>
-      <c r="B87" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="89" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A89" t="s">
-        <v>115</v>
-      </c>
-      <c r="B89">
-        <v>2</v>
-      </c>
-    </row>
+    <row r="89" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="90" spans="1:3" ht="14.25" customHeight="1">
       <c r="A90" t="s">
-        <v>116</v>
-      </c>
-      <c r="B90">
-        <v>40000</v>
-      </c>
-      <c r="C90" t="s">
-        <v>72</v>
+        <v>109</v>
+      </c>
+      <c r="B90" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="91" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A91" s="6"/>
-      <c r="B91" s="7"/>
-    </row>
-    <row r="92" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A92" t="s">
-        <v>106</v>
-      </c>
-      <c r="B92">
-        <v>30000</v>
-      </c>
-      <c r="C92" t="s">
-        <v>72</v>
-      </c>
-    </row>
+      <c r="A91" t="s">
+        <v>97</v>
+      </c>
+      <c r="B91" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="93" spans="1:3" ht="14.25" customHeight="1">
       <c r="A93" t="s">
-        <v>103</v>
-      </c>
-      <c r="B93">
-        <v>30000</v>
-      </c>
-      <c r="C93" t="s">
-        <v>72</v>
+        <v>111</v>
+      </c>
+      <c r="B93" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="94" spans="1:3" ht="14.25" customHeight="1">
       <c r="A94" t="s">
-        <v>107</v>
-      </c>
-      <c r="B94">
-        <v>60000</v>
-      </c>
-      <c r="C94" t="s">
-        <v>72</v>
+        <v>117</v>
+      </c>
+      <c r="B94" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="95" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A95" s="6"/>
-      <c r="B95" s="7"/>
-      <c r="C95" s="6"/>
+      <c r="A95" t="s">
+        <v>112</v>
+      </c>
+      <c r="B95" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="96" spans="1:3" ht="14.25" customHeight="1">
       <c r="A96" t="s">
-        <v>74</v>
-      </c>
-      <c r="B96">
-        <v>2000</v>
-      </c>
-      <c r="C96" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A97" t="s">
-        <v>76</v>
-      </c>
-      <c r="B97">
-        <v>10</v>
-      </c>
-    </row>
+        <v>118</v>
+      </c>
+      <c r="B96" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="98" spans="1:3" ht="14.25" customHeight="1">
       <c r="A98" t="s">
-        <v>77</v>
+        <v>244</v>
       </c>
       <c r="B98">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C98" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
     </row>
     <row r="99" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="100" spans="1:3" ht="15" customHeight="1">
+    <row r="100" spans="1:3" ht="14.25" customHeight="1">
       <c r="A100" t="s">
-        <v>75</v>
+        <v>115</v>
       </c>
       <c r="B100">
-        <v>2000</v>
-      </c>
-      <c r="C100" t="s">
-        <v>72</v>
+        <v>2</v>
       </c>
     </row>
     <row r="101" spans="1:3" ht="14.25" customHeight="1">
       <c r="A101" t="s">
-        <v>78</v>
+        <v>116</v>
       </c>
       <c r="B101">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" ht="17.5" customHeight="1">
-      <c r="A102" t="s">
-        <v>79</v>
-      </c>
-      <c r="B102">
-        <v>1</v>
-      </c>
-      <c r="C102" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" ht="17.5" customHeight="1"/>
-    <row r="104" spans="1:3" ht="17.5" customHeight="1">
+        <v>40000</v>
+      </c>
+      <c r="C101" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A102" s="6"/>
+      <c r="B102" s="7"/>
+    </row>
+    <row r="103" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A103" t="s">
+        <v>106</v>
+      </c>
+      <c r="B103">
+        <v>30000</v>
+      </c>
+      <c r="C103" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" ht="14.25" customHeight="1">
       <c r="A104" t="s">
-        <v>151</v>
+        <v>103</v>
       </c>
       <c r="B104">
-        <v>3000</v>
+        <v>30000</v>
       </c>
       <c r="C104" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="105" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A105" t="s">
+        <v>107</v>
+      </c>
+      <c r="B105">
+        <v>60000</v>
+      </c>
+      <c r="C105" t="s">
+        <v>72</v>
+      </c>
+    </row>
     <row r="106" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A106" t="s">
-        <v>121</v>
-      </c>
-      <c r="B106" t="s">
-        <v>346</v>
-      </c>
+      <c r="A106" s="6"/>
+      <c r="B106" s="7"/>
+      <c r="C106" s="6"/>
     </row>
     <row r="107" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A107" s="6"/>
-      <c r="B107" s="7"/>
-      <c r="C107" s="6"/>
-    </row>
-    <row r="108" spans="1:3" ht="14" customHeight="1">
+      <c r="A107" t="s">
+        <v>74</v>
+      </c>
+      <c r="B107">
+        <v>2000</v>
+      </c>
+      <c r="C107" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" ht="14.25" customHeight="1">
       <c r="A108" t="s">
-        <v>122</v>
+        <v>76</v>
       </c>
       <c r="B108">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A109" t="s">
+        <v>77</v>
+      </c>
+      <c r="B109">
         <v>1</v>
       </c>
-      <c r="C108" t="s">
+      <c r="C109" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="109" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="110" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A110" t="s">
-        <v>134</v>
-      </c>
-      <c r="B110">
-        <v>60000</v>
-      </c>
-      <c r="C110" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" ht="14.25" customHeight="1">
+    <row r="110" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="111" spans="1:3" ht="15" customHeight="1">
       <c r="A111" t="s">
-        <v>133</v>
+        <v>75</v>
       </c>
       <c r="B111">
-        <v>60000</v>
+        <v>2000</v>
       </c>
       <c r="C111" t="s">
         <v>72</v>
@@ -2319,319 +2033,309 @@
     </row>
     <row r="112" spans="1:3" ht="14.25" customHeight="1">
       <c r="A112" t="s">
+        <v>78</v>
+      </c>
+      <c r="B112">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" ht="17.5" customHeight="1">
+      <c r="A113" t="s">
+        <v>79</v>
+      </c>
+      <c r="B113">
+        <v>1</v>
+      </c>
+      <c r="C113" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" ht="17.5" customHeight="1"/>
+    <row r="115" spans="1:3" ht="17.5" customHeight="1">
+      <c r="A115" t="s">
+        <v>150</v>
+      </c>
+      <c r="B115">
+        <v>3000</v>
+      </c>
+      <c r="C115" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="117" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A117" t="s">
+        <v>121</v>
+      </c>
+      <c r="B117" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A118" s="6"/>
+      <c r="B118" s="7"/>
+      <c r="C118" s="6"/>
+    </row>
+    <row r="119" spans="1:3" ht="14" customHeight="1">
+      <c r="A119" t="s">
+        <v>122</v>
+      </c>
+      <c r="B119">
+        <v>1</v>
+      </c>
+      <c r="C119" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="121" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A121" t="s">
+        <v>133</v>
+      </c>
+      <c r="B121">
+        <v>60000</v>
+      </c>
+      <c r="C121" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A122" t="s">
+        <v>132</v>
+      </c>
+      <c r="B122">
+        <v>60000</v>
+      </c>
+      <c r="C122" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A123" t="s">
+        <v>134</v>
+      </c>
+      <c r="B123">
+        <v>60000</v>
+      </c>
+      <c r="C123" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A124" t="s">
+        <v>162</v>
+      </c>
+      <c r="B124">
+        <v>5</v>
+      </c>
+      <c r="C124" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="126" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A126" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B126" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A127" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B127" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A128" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B128" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A129" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B129" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" s="6" customFormat="1" ht="14.5"/>
+    <row r="131" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A131" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B131" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A132" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B132" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="A133" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B133" s="7">
+        <v>60</v>
+      </c>
+      <c r="C133" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="135" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A135" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B135" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C135" s="6"/>
+    </row>
+    <row r="136" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A136" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B136" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C136" s="6"/>
+    </row>
+    <row r="137" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A137" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B137" s="7">
+        <v>60</v>
+      </c>
+      <c r="C137" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A138" s="6"/>
+      <c r="B138" s="6"/>
+      <c r="C138" s="6"/>
+    </row>
+    <row r="139" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A139" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="B112">
+      <c r="B139" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C139" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A140" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="B140" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="C140" s="6"/>
+    </row>
+    <row r="141" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A141" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B141" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="C141" s="6"/>
+    </row>
+    <row r="142" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A142" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B142" s="6"/>
+      <c r="C142" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A143" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B143" s="7">
         <v>60000</v>
       </c>
-      <c r="C112" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A113" t="s">
-        <v>269</v>
-      </c>
-      <c r="B113">
-        <v>5</v>
-      </c>
-      <c r="C113" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="115" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A115" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B115" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A116" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B116" s="7" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A117" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B117" s="7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A118" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B118" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" s="6" customFormat="1" ht="14.5"/>
-    <row r="120" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A120" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B120" s="7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A121" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B121" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A122" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B122" s="7">
-        <v>60</v>
-      </c>
-      <c r="C122" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="124" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A124" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B124" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C124" s="6"/>
-    </row>
-    <row r="125" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A125" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B125" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C125" s="6"/>
-    </row>
-    <row r="126" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A126" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B126" s="7">
-        <v>60</v>
-      </c>
-      <c r="C126" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A127" s="6"/>
-      <c r="B127" s="6"/>
-      <c r="C127" s="6"/>
-    </row>
-    <row r="128" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A128" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="B128" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="C128" s="6" t="s">
+      <c r="C143" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="145" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A145" t="s">
+        <v>138</v>
+      </c>
+      <c r="B145" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C145" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="129" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A129" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B129" s="7" t="s">
-        <v>324</v>
-      </c>
-      <c r="C129" s="6"/>
-    </row>
-    <row r="130" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A130" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="B130" s="8" t="s">
-        <v>325</v>
-      </c>
-      <c r="C130" s="6"/>
-    </row>
-    <row r="131" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A131" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B131" s="6"/>
-      <c r="C131" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A132" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B132" s="7">
-        <v>60000</v>
-      </c>
-      <c r="C132" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="134" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A134" t="s">
-        <v>139</v>
-      </c>
-      <c r="B134" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="C134" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A135" t="s">
-        <v>140</v>
-      </c>
-      <c r="B135" s="7" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A136" t="s">
-        <v>141</v>
-      </c>
-      <c r="B136" s="8" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="137" spans="1:3" ht="14" customHeight="1"/>
-    <row r="138" spans="1:3" ht="14" customHeight="1">
-      <c r="A138" t="s">
-        <v>212</v>
-      </c>
-      <c r="B138" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" ht="14" customHeight="1">
-      <c r="A139" t="s">
-        <v>271</v>
-      </c>
-      <c r="B139" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" ht="14" customHeight="1">
-      <c r="A140" t="s">
-        <v>273</v>
-      </c>
-      <c r="B140" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3" ht="14" customHeight="1"/>
-    <row r="142" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A142" t="s">
-        <v>289</v>
-      </c>
-      <c r="B142" s="2">
-        <v>5</v>
-      </c>
-      <c r="C142" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A143" t="s">
-        <v>290</v>
-      </c>
-      <c r="B143" s="2">
-        <v>5</v>
-      </c>
-      <c r="C143" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A144" t="s">
-        <v>293</v>
-      </c>
-      <c r="B144" s="2">
-        <v>5</v>
-      </c>
-      <c r="C144" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="146" spans="1:3" ht="14.25" customHeight="1">
       <c r="A146" t="s">
-        <v>291</v>
-      </c>
-      <c r="B146" t="s">
-        <v>295</v>
+        <v>139</v>
+      </c>
+      <c r="B146" s="7" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="147" spans="1:3" ht="14.25" customHeight="1">
       <c r="A147" t="s">
-        <v>292</v>
-      </c>
-      <c r="B147" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="148" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A148" t="s">
-        <v>294</v>
-      </c>
-      <c r="B148" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3" ht="14.25" customHeight="1">
+        <v>140</v>
+      </c>
+      <c r="B147" s="8" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" ht="14" customHeight="1"/>
+    <row r="149" spans="1:3" ht="14" customHeight="1">
       <c r="A149" t="s">
-        <v>310</v>
+        <v>159</v>
       </c>
       <c r="B149" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3" ht="15.5" customHeight="1"/>
-    <row r="151" spans="1:3" ht="14.25" customHeight="1">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" ht="14" customHeight="1">
+      <c r="A150" t="s">
+        <v>163</v>
+      </c>
+      <c r="B150" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" ht="14" customHeight="1">
       <c r="A151" t="s">
-        <v>298</v>
-      </c>
-      <c r="B151">
-        <v>5</v>
-      </c>
-      <c r="C151" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="152" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A152" t="s">
-        <v>347</v>
-      </c>
-      <c r="B152">
-        <v>5</v>
-      </c>
-      <c r="C152" t="s">
-        <v>48</v>
-      </c>
-    </row>
+        <v>165</v>
+      </c>
+      <c r="B151" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" ht="14" customHeight="1"/>
     <row r="153" spans="1:3" ht="14.25" customHeight="1">
       <c r="A153" t="s">
-        <v>350</v>
-      </c>
-      <c r="B153">
+        <v>178</v>
+      </c>
+      <c r="B153" s="2">
         <v>5</v>
       </c>
       <c r="C153" t="s">
@@ -2640,186 +2344,308 @@
     </row>
     <row r="154" spans="1:3" ht="14.25" customHeight="1">
       <c r="A154" t="s">
-        <v>299</v>
-      </c>
-      <c r="B154" t="s">
-        <v>300</v>
+        <v>179</v>
+      </c>
+      <c r="B154" s="2">
+        <v>5</v>
+      </c>
+      <c r="C154" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="155" spans="1:3" ht="14.25" customHeight="1">
       <c r="A155" t="s">
-        <v>354</v>
-      </c>
-      <c r="B155" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="156" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A156" t="s">
-        <v>356</v>
-      </c>
-      <c r="B156" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="157" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="158" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="159" spans="1:3" ht="14.25" customHeight="1"/>
+        <v>182</v>
+      </c>
+      <c r="B155" s="2">
+        <v>5</v>
+      </c>
+      <c r="C155" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="157" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A157" t="s">
+        <v>180</v>
+      </c>
+      <c r="B157" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A158" t="s">
+        <v>181</v>
+      </c>
+      <c r="B158" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A159" t="s">
+        <v>183</v>
+      </c>
+      <c r="B159" t="s">
+        <v>186</v>
+      </c>
+    </row>
     <row r="160" spans="1:3" ht="14.25" customHeight="1">
       <c r="A160" t="s">
-        <v>301</v>
-      </c>
-      <c r="B160">
+        <v>199</v>
+      </c>
+      <c r="B160" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" ht="15.5" customHeight="1"/>
+    <row r="162" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A162" t="s">
+        <v>187</v>
+      </c>
+      <c r="B162">
         <v>5</v>
       </c>
-      <c r="C160" t="s">
+      <c r="C162" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="161" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A161" t="s">
-        <v>351</v>
-      </c>
-      <c r="B161">
-        <v>5</v>
-      </c>
-      <c r="C161" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="162" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="163" spans="1:3" ht="14.25" customHeight="1">
       <c r="A163" t="s">
-        <v>348</v>
-      </c>
-      <c r="B163" t="s">
-        <v>349</v>
+        <v>236</v>
+      </c>
+      <c r="B163">
+        <v>5</v>
+      </c>
+      <c r="C163" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="164" spans="1:3" ht="14.25" customHeight="1">
       <c r="A164" t="s">
-        <v>352</v>
-      </c>
-      <c r="B164" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="165" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="166" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="167" spans="1:3" ht="14.25" customHeight="1"/>
+        <v>239</v>
+      </c>
+      <c r="B164">
+        <v>5</v>
+      </c>
+      <c r="C164" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A165" t="s">
+        <v>188</v>
+      </c>
+      <c r="B165" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A166" t="s">
+        <v>241</v>
+      </c>
+      <c r="B166" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A167" t="s">
+        <v>243</v>
+      </c>
+      <c r="B167" t="s">
+        <v>238</v>
+      </c>
+    </row>
     <row r="168" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="169" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="170" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="171" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="172" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="173" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="174" spans="1:3" s="6" customFormat="1" ht="14.5"/>
-    <row r="175" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B175" s="7"/>
-    </row>
-    <row r="176" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B176" s="7"/>
-    </row>
-    <row r="177" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B177" s="7"/>
-    </row>
-    <row r="178" spans="1:3" s="6" customFormat="1" ht="14.5"/>
-    <row r="179" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B179" s="7"/>
-    </row>
-    <row r="180" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B180" s="7"/>
-    </row>
-    <row r="181" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="B181" s="7"/>
-    </row>
-    <row r="182" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="183" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A183" s="6"/>
-      <c r="B183" s="7"/>
-      <c r="C183" s="6"/>
-    </row>
-    <row r="184" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A184" s="6"/>
-      <c r="B184" s="8"/>
-      <c r="C184" s="6"/>
-    </row>
-    <row r="185" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A185" s="6"/>
-      <c r="B185" s="7"/>
-      <c r="C185" s="6"/>
-    </row>
-    <row r="186" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A186" s="6"/>
-      <c r="B186" s="6"/>
-      <c r="C186" s="6"/>
-    </row>
-    <row r="187" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A187" s="6"/>
-      <c r="B187" s="5"/>
-      <c r="C187" s="6"/>
-    </row>
-    <row r="188" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A188" s="6"/>
-      <c r="B188" s="7"/>
-      <c r="C188" s="6"/>
-    </row>
-    <row r="189" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A189" s="6"/>
-      <c r="B189" s="8"/>
-      <c r="C189" s="6"/>
-    </row>
-    <row r="190" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A190" s="6"/>
-      <c r="B190" s="6"/>
-      <c r="C190" s="6"/>
-    </row>
-    <row r="191" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A191" s="6"/>
+    <row r="171" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A171" t="s">
+        <v>190</v>
+      </c>
+      <c r="B171">
+        <v>5</v>
+      </c>
+      <c r="C171" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A172" t="s">
+        <v>240</v>
+      </c>
+      <c r="B172">
+        <v>5</v>
+      </c>
+      <c r="C172" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A173" t="s">
+        <v>257</v>
+      </c>
+      <c r="B173">
+        <v>5</v>
+      </c>
+      <c r="C173" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A174" t="s">
+        <v>260</v>
+      </c>
+      <c r="B174">
+        <v>5</v>
+      </c>
+      <c r="C174" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A175" t="s">
+        <v>263</v>
+      </c>
+      <c r="B175">
+        <v>5</v>
+      </c>
+      <c r="C175" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="177" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="178" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A178" t="s">
+        <v>237</v>
+      </c>
+      <c r="B178" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A179" t="s">
+        <v>264</v>
+      </c>
+      <c r="B179" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A180" t="s">
+        <v>258</v>
+      </c>
+      <c r="B180" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A181" t="s">
+        <v>261</v>
+      </c>
+      <c r="B181" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="183" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="184" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="185" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="186" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="187" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="188" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="189" spans="1:2" s="6" customFormat="1" ht="14.5"/>
+    <row r="190" spans="1:2" s="6" customFormat="1" ht="14.5">
+      <c r="B190" s="7"/>
+    </row>
+    <row r="191" spans="1:2" s="6" customFormat="1" ht="14.5">
       <c r="B191" s="7"/>
-      <c r="C191" s="6"/>
-    </row>
-    <row r="192" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="193" spans="1:2" ht="14.25" customHeight="1">
-      <c r="B193" s="5"/>
-    </row>
-    <row r="194" spans="1:2" ht="14.25" customHeight="1">
+    </row>
+    <row r="192" spans="1:2" s="6" customFormat="1" ht="14.5">
+      <c r="B192" s="7"/>
+    </row>
+    <row r="193" spans="1:3" s="6" customFormat="1" ht="14.5"/>
+    <row r="194" spans="1:3" s="6" customFormat="1" ht="14.5">
       <c r="B194" s="7"/>
     </row>
-    <row r="195" spans="1:2" ht="14.25" customHeight="1">
-      <c r="B195" s="8"/>
-    </row>
-    <row r="196" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="197" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A197" s="6"/>
-    </row>
-    <row r="198" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="199" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="200" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="201" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="202" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="203" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="204" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="205" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="206" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="207" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="208" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="209" ht="14.25" customHeight="1"/>
-    <row r="210" ht="14.25" customHeight="1"/>
-    <row r="211" ht="14.25" customHeight="1"/>
-    <row r="212" ht="14.25" customHeight="1"/>
-    <row r="213" ht="14.25" customHeight="1"/>
-    <row r="214" ht="14.25" customHeight="1"/>
-    <row r="215" ht="14.25" customHeight="1"/>
-    <row r="216" ht="14.25" customHeight="1"/>
-    <row r="217" ht="14.25" customHeight="1"/>
-    <row r="218" ht="14.25" customHeight="1"/>
-    <row r="219" ht="14.25" customHeight="1"/>
-    <row r="220" ht="14.25" customHeight="1"/>
-    <row r="221" ht="14.25" customHeight="1"/>
-    <row r="222" ht="14.25" customHeight="1"/>
-    <row r="223" ht="14.25" customHeight="1"/>
-    <row r="224" ht="14.25" customHeight="1"/>
+    <row r="195" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B195" s="7"/>
+    </row>
+    <row r="196" spans="1:3" s="6" customFormat="1" ht="14.5">
+      <c r="B196" s="7"/>
+    </row>
+    <row r="197" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="198" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A198" s="6"/>
+      <c r="B198" s="7"/>
+      <c r="C198" s="6"/>
+    </row>
+    <row r="199" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A199" s="6"/>
+      <c r="B199" s="8"/>
+      <c r="C199" s="6"/>
+    </row>
+    <row r="200" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A200" s="6"/>
+      <c r="B200" s="7"/>
+      <c r="C200" s="6"/>
+    </row>
+    <row r="201" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A201" s="6"/>
+      <c r="B201" s="6"/>
+      <c r="C201" s="6"/>
+    </row>
+    <row r="202" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A202" s="6"/>
+      <c r="B202" s="5"/>
+      <c r="C202" s="6"/>
+    </row>
+    <row r="203" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A203" s="6"/>
+      <c r="B203" s="7"/>
+      <c r="C203" s="6"/>
+    </row>
+    <row r="204" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A204" s="6"/>
+      <c r="B204" s="8"/>
+      <c r="C204" s="6"/>
+    </row>
+    <row r="205" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A205" s="6"/>
+      <c r="B205" s="6"/>
+      <c r="C205" s="6"/>
+    </row>
+    <row r="206" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A206" s="6"/>
+      <c r="B206" s="7"/>
+      <c r="C206" s="6"/>
+    </row>
+    <row r="207" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="208" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B208" s="5"/>
+    </row>
+    <row r="209" spans="1:2" ht="14.25" customHeight="1">
+      <c r="B209" s="7"/>
+    </row>
+    <row r="210" spans="1:2" ht="14.25" customHeight="1">
+      <c r="B210" s="8"/>
+    </row>
+    <row r="211" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="212" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A212" s="6"/>
+    </row>
+    <row r="213" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="214" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="215" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="216" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="217" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="218" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="219" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="220" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="221" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="222" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="223" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="224" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="225" ht="14.25" customHeight="1"/>
     <row r="226" ht="14.25" customHeight="1"/>
     <row r="227" ht="14.25" customHeight="1"/>
@@ -3649,6 +3475,21 @@
     <row r="1051" ht="14.25" customHeight="1"/>
     <row r="1052" ht="14.25" customHeight="1"/>
     <row r="1053" ht="14.25" customHeight="1"/>
+    <row r="1054" ht="14.25" customHeight="1"/>
+    <row r="1055" ht="14.25" customHeight="1"/>
+    <row r="1056" ht="14.25" customHeight="1"/>
+    <row r="1057" ht="14.25" customHeight="1"/>
+    <row r="1058" ht="14.25" customHeight="1"/>
+    <row r="1059" ht="14.25" customHeight="1"/>
+    <row r="1060" ht="14.25" customHeight="1"/>
+    <row r="1061" ht="14.25" customHeight="1"/>
+    <row r="1062" ht="14.25" customHeight="1"/>
+    <row r="1063" ht="14.25" customHeight="1"/>
+    <row r="1064" ht="14.25" customHeight="1"/>
+    <row r="1065" ht="14.25" customHeight="1"/>
+    <row r="1066" ht="14.25" customHeight="1"/>
+    <row r="1067" ht="14.25" customHeight="1"/>
+    <row r="1068" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3843,7 +3684,7 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>343</v>
+        <v>232</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1"/>
@@ -5875,2276 +5716,4 @@
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E2E1777-460A-49FA-8ECC-5B7815DCE559}">
-  <dimension ref="A1:Z1079"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="49.54296875" customWidth="1"/>
-    <col min="2" max="2" width="72.7265625" customWidth="1"/>
-    <col min="3" max="3" width="22.6328125" customWidth="1"/>
-    <col min="4" max="26" width="8.6328125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
-    </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:26" ht="15" customHeight="1">
-      <c r="A3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B3" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A4" t="s">
-        <v>81</v>
-      </c>
-      <c r="B4">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" ht="14.5">
-      <c r="A5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B5">
-        <v>1000</v>
-      </c>
-      <c r="C5" s="4"/>
-    </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" t="s">
-        <v>83</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" t="s">
-        <v>84</v>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="B8" s="9">
-        <v>0</v>
-      </c>
-      <c r="C8" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-    </row>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A12" t="s">
-        <v>153</v>
-      </c>
-      <c r="B12" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26" ht="15" customHeight="1">
-      <c r="A13" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A14" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" spans="1:26" ht="15" customHeight="1">
-      <c r="A15" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" ht="15" customHeight="1">
-      <c r="A16" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="15" customHeight="1">
-      <c r="A17" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="15" customHeight="1">
-      <c r="A18" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="15" customHeight="1">
-      <c r="A19" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="15" customHeight="1">
-      <c r="A20" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="15" customHeight="1">
-      <c r="A21" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="15" customHeight="1">
-      <c r="A22" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="14.5">
-      <c r="A23" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="14.5">
-      <c r="A24" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="14.5">
-      <c r="A26" t="s">
-        <v>205</v>
-      </c>
-      <c r="B26" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="15" customHeight="1">
-      <c r="A27" t="s">
-        <v>163</v>
-      </c>
-      <c r="B27" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="14.5">
-      <c r="A28" t="s">
-        <v>164</v>
-      </c>
-      <c r="B28" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="14.5">
-      <c r="A29" t="s">
-        <v>172</v>
-      </c>
-      <c r="B29" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="14.5">
-      <c r="A30" t="s">
-        <v>173</v>
-      </c>
-      <c r="B30" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="14.5">
-      <c r="A31" t="s">
-        <v>174</v>
-      </c>
-      <c r="B31" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="33" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A33" t="s">
-        <v>129</v>
-      </c>
-      <c r="B33" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A34" t="s">
-        <v>67</v>
-      </c>
-      <c r="B34" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="36" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A36" t="s">
-        <v>49</v>
-      </c>
-      <c r="B36" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A37" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="15" customHeight="1">
-      <c r="A39" t="s">
-        <v>63</v>
-      </c>
-      <c r="B39" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="15" customHeight="1">
-      <c r="A40" t="s">
-        <v>64</v>
-      </c>
-      <c r="B40" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="15" customHeight="1">
-      <c r="A41" t="s">
-        <v>65</v>
-      </c>
-      <c r="B41" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A43" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="B43" s="11" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="14.5">
-      <c r="A44" t="s">
-        <v>156</v>
-      </c>
-      <c r="B44" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="14.5">
-      <c r="A45" t="s">
-        <v>180</v>
-      </c>
-      <c r="B45" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" ht="14.5">
-      <c r="A46" t="s">
-        <v>178</v>
-      </c>
-      <c r="B46" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" ht="14.5">
-      <c r="A47" t="s">
-        <v>182</v>
-      </c>
-      <c r="B47" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" ht="14.5">
-      <c r="A48" t="s">
-        <v>184</v>
-      </c>
-      <c r="B48" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="14.5">
-      <c r="A49" t="s">
-        <v>145</v>
-      </c>
-      <c r="B49" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" ht="14.5">
-      <c r="A50" t="s">
-        <v>147</v>
-      </c>
-      <c r="B50" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="14.5">
-      <c r="A51" t="s">
-        <v>94</v>
-      </c>
-      <c r="B51" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" ht="14.5">
-      <c r="A52" t="s">
-        <v>149</v>
-      </c>
-      <c r="B52" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" ht="14.5">
-      <c r="A53" t="s">
-        <v>188</v>
-      </c>
-      <c r="B53" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="14.5">
-      <c r="A54" t="s">
-        <v>190</v>
-      </c>
-      <c r="B54" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A55" t="s">
-        <v>123</v>
-      </c>
-      <c r="B55" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A56" t="s">
-        <v>124</v>
-      </c>
-      <c r="B56" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A57" t="s">
-        <v>220</v>
-      </c>
-      <c r="B57" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A58" t="s">
-        <v>223</v>
-      </c>
-      <c r="B58" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" ht="14.5">
-      <c r="A59" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" ht="14.5">
-      <c r="A60" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" ht="14.5">
-      <c r="A61" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" ht="14.5">
-      <c r="A62" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" ht="14.5">
-      <c r="A63" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" ht="14.5">
-      <c r="A64" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" ht="14.5">
-      <c r="A65" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" ht="14.5">
-      <c r="A66" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" ht="14.5">
-      <c r="A67" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" ht="14.5">
-      <c r="A68" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" ht="14.5">
-      <c r="A69" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" ht="14.5">
-      <c r="A70" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" ht="14.5">
-      <c r="A71" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" ht="14.5">
-      <c r="A72" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" ht="14.5">
-      <c r="A73" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" ht="14.5">
-      <c r="A74" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" ht="14.5">
-      <c r="A75" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" ht="14.5">
-      <c r="A76" s="2"/>
-      <c r="B76" s="2"/>
-    </row>
-    <row r="77" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A77" t="s">
-        <v>88</v>
-      </c>
-      <c r="B77" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A78" t="s">
-        <v>95</v>
-      </c>
-      <c r="B78" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A79" t="s">
-        <v>89</v>
-      </c>
-      <c r="B79" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A80" t="s">
-        <v>104</v>
-      </c>
-      <c r="B80" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A81" t="s">
-        <v>108</v>
-      </c>
-      <c r="B81" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A82" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A83" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="B83" s="9" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" s="9" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A84" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="B84" s="9" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A85" s="2"/>
-      <c r="B85" s="2"/>
-    </row>
-    <row r="86" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A86" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B86" s="7">
-        <v>2000</v>
-      </c>
-      <c r="C86" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A87" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B87">
-        <v>1</v>
-      </c>
-      <c r="C87" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A88" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B88" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="C88" s="6"/>
-    </row>
-    <row r="89" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A89" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="B89" s="7">
-        <v>3</v>
-      </c>
-      <c r="C89" s="6"/>
-    </row>
-    <row r="90" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A90" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B90" s="7">
-        <v>3</v>
-      </c>
-      <c r="C90" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" ht="14.5"/>
-    <row r="92" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A92" t="s">
-        <v>91</v>
-      </c>
-      <c r="B92" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="94" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A94" t="s">
-        <v>109</v>
-      </c>
-      <c r="B94" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A95" t="s">
-        <v>97</v>
-      </c>
-      <c r="B95" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="97" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A97" t="s">
-        <v>111</v>
-      </c>
-      <c r="B97" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A98" t="s">
-        <v>117</v>
-      </c>
-      <c r="B98" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A99" t="s">
-        <v>112</v>
-      </c>
-      <c r="B99" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A100" t="s">
-        <v>118</v>
-      </c>
-      <c r="B100" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="102" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A102" t="s">
-        <v>115</v>
-      </c>
-      <c r="B102">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A103" t="s">
-        <v>116</v>
-      </c>
-      <c r="B103">
-        <v>40000</v>
-      </c>
-      <c r="C103" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A104" s="6"/>
-      <c r="B104" s="7"/>
-    </row>
-    <row r="105" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A105" t="s">
-        <v>106</v>
-      </c>
-      <c r="B105">
-        <v>30000</v>
-      </c>
-      <c r="C105" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A106" t="s">
-        <v>103</v>
-      </c>
-      <c r="B106">
-        <v>30000</v>
-      </c>
-      <c r="C106" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A107" t="s">
-        <v>107</v>
-      </c>
-      <c r="B107">
-        <v>60000</v>
-      </c>
-      <c r="C107" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A108" s="6"/>
-      <c r="B108" s="7"/>
-      <c r="C108" s="6"/>
-    </row>
-    <row r="109" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A109" t="s">
-        <v>74</v>
-      </c>
-      <c r="B109">
-        <v>2000</v>
-      </c>
-      <c r="C109" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A110" t="s">
-        <v>76</v>
-      </c>
-      <c r="B110">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A111" t="s">
-        <v>77</v>
-      </c>
-      <c r="B111">
-        <v>1</v>
-      </c>
-      <c r="C111" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="113" spans="1:3" ht="15" customHeight="1">
-      <c r="A113" t="s">
-        <v>75</v>
-      </c>
-      <c r="B113">
-        <v>2000</v>
-      </c>
-      <c r="C113" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A114" t="s">
-        <v>78</v>
-      </c>
-      <c r="B114">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" ht="17.5" customHeight="1">
-      <c r="A115" t="s">
-        <v>79</v>
-      </c>
-      <c r="B115">
-        <v>1</v>
-      </c>
-      <c r="C115" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" ht="17.5" customHeight="1"/>
-    <row r="117" spans="1:3" ht="17.5" customHeight="1">
-      <c r="A117" t="s">
-        <v>151</v>
-      </c>
-      <c r="B117">
-        <v>3000</v>
-      </c>
-      <c r="C117" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="119" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A119" t="s">
-        <v>121</v>
-      </c>
-      <c r="B119" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A120" s="6"/>
-      <c r="B120" s="7"/>
-      <c r="C120" s="6"/>
-    </row>
-    <row r="121" spans="1:3" ht="14" customHeight="1">
-      <c r="A121" t="s">
-        <v>122</v>
-      </c>
-      <c r="B121">
-        <v>1</v>
-      </c>
-      <c r="C121" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="123" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A123" t="s">
-        <v>134</v>
-      </c>
-      <c r="B123">
-        <v>60000</v>
-      </c>
-      <c r="C123" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A124" t="s">
-        <v>133</v>
-      </c>
-      <c r="B124">
-        <v>60000</v>
-      </c>
-      <c r="C124" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A125" t="s">
-        <v>135</v>
-      </c>
-      <c r="B125">
-        <v>60000</v>
-      </c>
-      <c r="C125" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A126" t="s">
-        <v>269</v>
-      </c>
-      <c r="B126">
-        <v>5</v>
-      </c>
-      <c r="C126" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A127" t="s">
-        <v>270</v>
-      </c>
-      <c r="B127">
-        <v>5</v>
-      </c>
-      <c r="C127" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3" ht="14.5" customHeight="1">
-      <c r="A128" t="s">
-        <v>261</v>
-      </c>
-      <c r="B128">
-        <v>5</v>
-      </c>
-      <c r="C128" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="130" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A130" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="B130" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" ht="17.5" customHeight="1"/>
-    <row r="132" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A132" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B132" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A133" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B133" s="7" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A134" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B134" s="7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A135" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B135" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3" s="6" customFormat="1" ht="14.5"/>
-    <row r="137" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A137" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B137" s="7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A138" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B138" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" s="6" customFormat="1" ht="14.5">
-      <c r="A139" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B139" s="7">
-        <v>60</v>
-      </c>
-      <c r="C139" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="141" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A141" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B141" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C141" s="6"/>
-    </row>
-    <row r="142" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A142" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B142" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C142" s="6"/>
-    </row>
-    <row r="143" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A143" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B143" s="7">
-        <v>60</v>
-      </c>
-      <c r="C143" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A144" s="6"/>
-      <c r="B144" s="6"/>
-      <c r="C144" s="6"/>
-    </row>
-    <row r="145" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A145" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="B145" s="5" t="s">
-        <v>277</v>
-      </c>
-      <c r="C145" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="146" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A146" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B146" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="C146" s="6"/>
-    </row>
-    <row r="147" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A147" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="B147" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="C147" s="6"/>
-    </row>
-    <row r="148" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A148" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B148" s="6"/>
-      <c r="C148" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A149" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B149" s="7">
-        <v>60000</v>
-      </c>
-      <c r="C149" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="151" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A151" t="s">
-        <v>139</v>
-      </c>
-      <c r="B151" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="C151" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="152" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A152" t="s">
-        <v>140</v>
-      </c>
-      <c r="B152" s="7" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="153" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A153" t="s">
-        <v>141</v>
-      </c>
-      <c r="B153" s="8" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="154" spans="1:3" ht="14" customHeight="1"/>
-    <row r="155" spans="1:3" ht="14" customHeight="1">
-      <c r="A155" t="s">
-        <v>210</v>
-      </c>
-      <c r="B155">
-        <v>5</v>
-      </c>
-      <c r="C155" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="156" spans="1:3" ht="14" customHeight="1"/>
-    <row r="157" spans="1:3" ht="14" customHeight="1">
-      <c r="A157" t="s">
-        <v>212</v>
-      </c>
-      <c r="B157" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3" ht="14" customHeight="1">
-      <c r="A158" t="s">
-        <v>271</v>
-      </c>
-      <c r="B158" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="159" spans="1:3" ht="14" customHeight="1">
-      <c r="A159" t="s">
-        <v>273</v>
-      </c>
-      <c r="B159" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="160" spans="1:3" ht="14" customHeight="1"/>
-    <row r="161" spans="1:3" ht="14" customHeight="1">
-      <c r="A161" t="s">
-        <v>216</v>
-      </c>
-      <c r="B161" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="162" spans="1:3" ht="14" customHeight="1">
-      <c r="A162" t="s">
-        <v>217</v>
-      </c>
-      <c r="B162" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="163" spans="1:3" ht="14" customHeight="1"/>
-    <row r="164" spans="1:3" ht="15" customHeight="1">
-      <c r="A164" t="s">
-        <v>218</v>
-      </c>
-      <c r="B164" s="12" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="165" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A165" t="s">
-        <v>222</v>
-      </c>
-      <c r="B165" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="166" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A166" t="s">
-        <v>257</v>
-      </c>
-      <c r="B166" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A167" t="s">
-        <v>258</v>
-      </c>
-      <c r="B167" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="169" spans="1:3" ht="15" customHeight="1">
-      <c r="A169" t="s">
-        <v>262</v>
-      </c>
-      <c r="B169" s="12" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="170" spans="1:3" ht="15" customHeight="1">
-      <c r="A170" t="s">
-        <v>263</v>
-      </c>
-      <c r="B170" s="12" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="171" spans="1:3" ht="15" customHeight="1">
-      <c r="B171" s="12"/>
-    </row>
-    <row r="172" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A172" t="s">
-        <v>275</v>
-      </c>
-      <c r="B172" s="2">
-        <v>25</v>
-      </c>
-      <c r="C172" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="173" spans="1:3" ht="15" customHeight="1">
-      <c r="B173" s="2"/>
-    </row>
-    <row r="174" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B174" s="2"/>
-    </row>
-    <row r="175" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B175" s="2"/>
-    </row>
-    <row r="176" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="177" ht="14.25" customHeight="1"/>
-    <row r="178" ht="14.25" customHeight="1"/>
-    <row r="179" ht="14.25" customHeight="1"/>
-    <row r="180" ht="14.25" customHeight="1"/>
-    <row r="181" ht="14.25" customHeight="1"/>
-    <row r="182" ht="14.25" customHeight="1"/>
-    <row r="183" ht="14.25" customHeight="1"/>
-    <row r="184" ht="14.25" customHeight="1"/>
-    <row r="185" ht="14.25" customHeight="1"/>
-    <row r="186" ht="14.25" customHeight="1"/>
-    <row r="187" ht="14.25" customHeight="1"/>
-    <row r="188" ht="14.25" customHeight="1"/>
-    <row r="189" ht="14.25" customHeight="1"/>
-    <row r="190" ht="14.25" customHeight="1"/>
-    <row r="191" ht="14.25" customHeight="1"/>
-    <row r="192" ht="14.25" customHeight="1"/>
-    <row r="193" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="194" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="195" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="196" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="197" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="198" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="199" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="200" spans="2:2" s="6" customFormat="1" ht="14.5"/>
-    <row r="201" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B201" s="7"/>
-    </row>
-    <row r="202" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B202" s="7"/>
-    </row>
-    <row r="203" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B203" s="7"/>
-    </row>
-    <row r="204" spans="2:2" s="6" customFormat="1" ht="14.5"/>
-    <row r="205" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B205" s="7"/>
-    </row>
-    <row r="206" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B206" s="7"/>
-    </row>
-    <row r="207" spans="2:2" s="6" customFormat="1" ht="14.5">
-      <c r="B207" s="7"/>
-    </row>
-    <row r="208" spans="2:2" ht="14.25" customHeight="1"/>
-    <row r="209" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A209" s="6"/>
-      <c r="B209" s="7"/>
-      <c r="C209" s="6"/>
-    </row>
-    <row r="210" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A210" s="6"/>
-      <c r="B210" s="8"/>
-      <c r="C210" s="6"/>
-    </row>
-    <row r="211" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A211" s="6"/>
-      <c r="B211" s="7"/>
-      <c r="C211" s="6"/>
-    </row>
-    <row r="212" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A212" s="6"/>
-      <c r="B212" s="6"/>
-      <c r="C212" s="6"/>
-    </row>
-    <row r="213" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A213" s="6"/>
-      <c r="B213" s="5"/>
-      <c r="C213" s="6"/>
-    </row>
-    <row r="214" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A214" s="6"/>
-      <c r="B214" s="7"/>
-      <c r="C214" s="6"/>
-    </row>
-    <row r="215" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A215" s="6"/>
-      <c r="B215" s="8"/>
-      <c r="C215" s="6"/>
-    </row>
-    <row r="216" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A216" s="6"/>
-      <c r="B216" s="6"/>
-      <c r="C216" s="6"/>
-    </row>
-    <row r="217" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A217" s="6"/>
-      <c r="B217" s="7"/>
-      <c r="C217" s="6"/>
-    </row>
-    <row r="218" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="219" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B219" s="5"/>
-    </row>
-    <row r="220" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B220" s="7"/>
-    </row>
-    <row r="221" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B221" s="8"/>
-    </row>
-    <row r="222" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="223" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A223" s="6"/>
-    </row>
-    <row r="224" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="225" ht="14.25" customHeight="1"/>
-    <row r="226" ht="14.25" customHeight="1"/>
-    <row r="227" ht="14.25" customHeight="1"/>
-    <row r="228" ht="14.25" customHeight="1"/>
-    <row r="229" ht="14.25" customHeight="1"/>
-    <row r="230" ht="14.25" customHeight="1"/>
-    <row r="231" ht="14.25" customHeight="1"/>
-    <row r="232" ht="14.25" customHeight="1"/>
-    <row r="233" ht="14.25" customHeight="1"/>
-    <row r="234" ht="14.25" customHeight="1"/>
-    <row r="235" ht="14.25" customHeight="1"/>
-    <row r="236" ht="14.25" customHeight="1"/>
-    <row r="237" ht="14.25" customHeight="1"/>
-    <row r="238" ht="14.25" customHeight="1"/>
-    <row r="239" ht="14.25" customHeight="1"/>
-    <row r="240" ht="14.25" customHeight="1"/>
-    <row r="241" ht="14.25" customHeight="1"/>
-    <row r="242" ht="14.25" customHeight="1"/>
-    <row r="243" ht="14.25" customHeight="1"/>
-    <row r="244" ht="14.25" customHeight="1"/>
-    <row r="245" ht="14.25" customHeight="1"/>
-    <row r="246" ht="14.25" customHeight="1"/>
-    <row r="247" ht="14.25" customHeight="1"/>
-    <row r="248" ht="14.25" customHeight="1"/>
-    <row r="249" ht="14.25" customHeight="1"/>
-    <row r="250" ht="14.25" customHeight="1"/>
-    <row r="251" ht="14.25" customHeight="1"/>
-    <row r="252" ht="14.25" customHeight="1"/>
-    <row r="253" ht="14.25" customHeight="1"/>
-    <row r="254" ht="14.25" customHeight="1"/>
-    <row r="255" ht="14.25" customHeight="1"/>
-    <row r="256" ht="14.25" customHeight="1"/>
-    <row r="257" ht="14.25" customHeight="1"/>
-    <row r="258" ht="14.25" customHeight="1"/>
-    <row r="259" ht="14.25" customHeight="1"/>
-    <row r="260" ht="14.25" customHeight="1"/>
-    <row r="261" ht="14.25" customHeight="1"/>
-    <row r="262" ht="14.25" customHeight="1"/>
-    <row r="263" ht="14.25" customHeight="1"/>
-    <row r="264" ht="14.25" customHeight="1"/>
-    <row r="265" ht="14.25" customHeight="1"/>
-    <row r="266" ht="14.25" customHeight="1"/>
-    <row r="267" ht="14.25" customHeight="1"/>
-    <row r="268" ht="14.25" customHeight="1"/>
-    <row r="269" ht="14.25" customHeight="1"/>
-    <row r="270" ht="14.25" customHeight="1"/>
-    <row r="271" ht="14.25" customHeight="1"/>
-    <row r="272" ht="14.25" customHeight="1"/>
-    <row r="273" ht="14.25" customHeight="1"/>
-    <row r="274" ht="14.25" customHeight="1"/>
-    <row r="275" ht="14.25" customHeight="1"/>
-    <row r="276" ht="14.25" customHeight="1"/>
-    <row r="277" ht="14.25" customHeight="1"/>
-    <row r="278" ht="14.25" customHeight="1"/>
-    <row r="279" ht="14.25" customHeight="1"/>
-    <row r="280" ht="14.25" customHeight="1"/>
-    <row r="281" ht="14.25" customHeight="1"/>
-    <row r="282" ht="14.25" customHeight="1"/>
-    <row r="283" ht="14.25" customHeight="1"/>
-    <row r="284" ht="14.25" customHeight="1"/>
-    <row r="285" ht="14.25" customHeight="1"/>
-    <row r="286" ht="14.25" customHeight="1"/>
-    <row r="287" ht="14.25" customHeight="1"/>
-    <row r="288" ht="14.25" customHeight="1"/>
-    <row r="289" ht="14.25" customHeight="1"/>
-    <row r="290" ht="14.25" customHeight="1"/>
-    <row r="291" ht="14.25" customHeight="1"/>
-    <row r="292" ht="14.25" customHeight="1"/>
-    <row r="293" ht="14.25" customHeight="1"/>
-    <row r="294" ht="14.25" customHeight="1"/>
-    <row r="295" ht="14.25" customHeight="1"/>
-    <row r="296" ht="14.25" customHeight="1"/>
-    <row r="297" ht="14.25" customHeight="1"/>
-    <row r="298" ht="14.25" customHeight="1"/>
-    <row r="299" ht="14.25" customHeight="1"/>
-    <row r="300" ht="14.25" customHeight="1"/>
-    <row r="301" ht="14.25" customHeight="1"/>
-    <row r="302" ht="14.25" customHeight="1"/>
-    <row r="303" ht="14.25" customHeight="1"/>
-    <row r="304" ht="14.25" customHeight="1"/>
-    <row r="305" ht="14.25" customHeight="1"/>
-    <row r="306" ht="14.25" customHeight="1"/>
-    <row r="307" ht="14.25" customHeight="1"/>
-    <row r="308" ht="14.25" customHeight="1"/>
-    <row r="309" ht="14.25" customHeight="1"/>
-    <row r="310" ht="14.25" customHeight="1"/>
-    <row r="311" ht="14.25" customHeight="1"/>
-    <row r="312" ht="14.25" customHeight="1"/>
-    <row r="313" ht="14.25" customHeight="1"/>
-    <row r="314" ht="14.25" customHeight="1"/>
-    <row r="315" ht="14.25" customHeight="1"/>
-    <row r="316" ht="14.25" customHeight="1"/>
-    <row r="317" ht="14.25" customHeight="1"/>
-    <row r="318" ht="14.25" customHeight="1"/>
-    <row r="319" ht="14.25" customHeight="1"/>
-    <row r="320" ht="14.25" customHeight="1"/>
-    <row r="321" ht="14.25" customHeight="1"/>
-    <row r="322" ht="14.25" customHeight="1"/>
-    <row r="323" ht="14.25" customHeight="1"/>
-    <row r="324" ht="14.25" customHeight="1"/>
-    <row r="325" ht="14.25" customHeight="1"/>
-    <row r="326" ht="14.25" customHeight="1"/>
-    <row r="327" ht="14.25" customHeight="1"/>
-    <row r="328" ht="14.25" customHeight="1"/>
-    <row r="329" ht="14.25" customHeight="1"/>
-    <row r="330" ht="14.25" customHeight="1"/>
-    <row r="331" ht="14.25" customHeight="1"/>
-    <row r="332" ht="14.25" customHeight="1"/>
-    <row r="333" ht="14.25" customHeight="1"/>
-    <row r="334" ht="14.25" customHeight="1"/>
-    <row r="335" ht="14.25" customHeight="1"/>
-    <row r="336" ht="14.25" customHeight="1"/>
-    <row r="337" ht="14.25" customHeight="1"/>
-    <row r="338" ht="14.25" customHeight="1"/>
-    <row r="339" ht="14.25" customHeight="1"/>
-    <row r="340" ht="14.25" customHeight="1"/>
-    <row r="341" ht="14.25" customHeight="1"/>
-    <row r="342" ht="14.25" customHeight="1"/>
-    <row r="343" ht="14.25" customHeight="1"/>
-    <row r="344" ht="14.25" customHeight="1"/>
-    <row r="345" ht="14.25" customHeight="1"/>
-    <row r="346" ht="14.25" customHeight="1"/>
-    <row r="347" ht="14.25" customHeight="1"/>
-    <row r="348" ht="14.25" customHeight="1"/>
-    <row r="349" ht="14.25" customHeight="1"/>
-    <row r="350" ht="14.25" customHeight="1"/>
-    <row r="351" ht="14.25" customHeight="1"/>
-    <row r="352" ht="14.25" customHeight="1"/>
-    <row r="353" ht="14.25" customHeight="1"/>
-    <row r="354" ht="14.25" customHeight="1"/>
-    <row r="355" ht="14.25" customHeight="1"/>
-    <row r="356" ht="14.25" customHeight="1"/>
-    <row r="357" ht="14.25" customHeight="1"/>
-    <row r="358" ht="14.25" customHeight="1"/>
-    <row r="359" ht="14.25" customHeight="1"/>
-    <row r="360" ht="14.25" customHeight="1"/>
-    <row r="361" ht="14.25" customHeight="1"/>
-    <row r="362" ht="14.25" customHeight="1"/>
-    <row r="363" ht="14.25" customHeight="1"/>
-    <row r="364" ht="14.25" customHeight="1"/>
-    <row r="365" ht="14.25" customHeight="1"/>
-    <row r="366" ht="14.25" customHeight="1"/>
-    <row r="367" ht="14.25" customHeight="1"/>
-    <row r="368" ht="14.25" customHeight="1"/>
-    <row r="369" ht="14.25" customHeight="1"/>
-    <row r="370" ht="14.25" customHeight="1"/>
-    <row r="371" ht="14.25" customHeight="1"/>
-    <row r="372" ht="14.25" customHeight="1"/>
-    <row r="373" ht="14.25" customHeight="1"/>
-    <row r="374" ht="14.25" customHeight="1"/>
-    <row r="375" ht="14.25" customHeight="1"/>
-    <row r="376" ht="14.25" customHeight="1"/>
-    <row r="377" ht="14.25" customHeight="1"/>
-    <row r="378" ht="14.25" customHeight="1"/>
-    <row r="379" ht="14.25" customHeight="1"/>
-    <row r="380" ht="14.25" customHeight="1"/>
-    <row r="381" ht="14.25" customHeight="1"/>
-    <row r="382" ht="14.25" customHeight="1"/>
-    <row r="383" ht="14.25" customHeight="1"/>
-    <row r="384" ht="14.25" customHeight="1"/>
-    <row r="385" ht="14.25" customHeight="1"/>
-    <row r="386" ht="14.25" customHeight="1"/>
-    <row r="387" ht="14.25" customHeight="1"/>
-    <row r="388" ht="14.25" customHeight="1"/>
-    <row r="389" ht="14.25" customHeight="1"/>
-    <row r="390" ht="14.25" customHeight="1"/>
-    <row r="391" ht="14.25" customHeight="1"/>
-    <row r="392" ht="14.25" customHeight="1"/>
-    <row r="393" ht="14.25" customHeight="1"/>
-    <row r="394" ht="14.25" customHeight="1"/>
-    <row r="395" ht="14.25" customHeight="1"/>
-    <row r="396" ht="14.25" customHeight="1"/>
-    <row r="397" ht="14.25" customHeight="1"/>
-    <row r="398" ht="14.25" customHeight="1"/>
-    <row r="399" ht="14.25" customHeight="1"/>
-    <row r="400" ht="14.25" customHeight="1"/>
-    <row r="401" ht="14.25" customHeight="1"/>
-    <row r="402" ht="14.25" customHeight="1"/>
-    <row r="403" ht="14.25" customHeight="1"/>
-    <row r="404" ht="14.25" customHeight="1"/>
-    <row r="405" ht="14.25" customHeight="1"/>
-    <row r="406" ht="14.25" customHeight="1"/>
-    <row r="407" ht="14.25" customHeight="1"/>
-    <row r="408" ht="14.25" customHeight="1"/>
-    <row r="409" ht="14.25" customHeight="1"/>
-    <row r="410" ht="14.25" customHeight="1"/>
-    <row r="411" ht="14.25" customHeight="1"/>
-    <row r="412" ht="14.25" customHeight="1"/>
-    <row r="413" ht="14.25" customHeight="1"/>
-    <row r="414" ht="14.25" customHeight="1"/>
-    <row r="415" ht="14.25" customHeight="1"/>
-    <row r="416" ht="14.25" customHeight="1"/>
-    <row r="417" ht="14.25" customHeight="1"/>
-    <row r="418" ht="14.25" customHeight="1"/>
-    <row r="419" ht="14.25" customHeight="1"/>
-    <row r="420" ht="14.25" customHeight="1"/>
-    <row r="421" ht="14.25" customHeight="1"/>
-    <row r="422" ht="14.25" customHeight="1"/>
-    <row r="423" ht="14.25" customHeight="1"/>
-    <row r="424" ht="14.25" customHeight="1"/>
-    <row r="425" ht="14.25" customHeight="1"/>
-    <row r="426" ht="14.25" customHeight="1"/>
-    <row r="427" ht="14.25" customHeight="1"/>
-    <row r="428" ht="14.25" customHeight="1"/>
-    <row r="429" ht="14.25" customHeight="1"/>
-    <row r="430" ht="14.25" customHeight="1"/>
-    <row r="431" ht="14.25" customHeight="1"/>
-    <row r="432" ht="14.25" customHeight="1"/>
-    <row r="433" ht="14.25" customHeight="1"/>
-    <row r="434" ht="14.25" customHeight="1"/>
-    <row r="435" ht="14.25" customHeight="1"/>
-    <row r="436" ht="14.25" customHeight="1"/>
-    <row r="437" ht="14.25" customHeight="1"/>
-    <row r="438" ht="14.25" customHeight="1"/>
-    <row r="439" ht="14.25" customHeight="1"/>
-    <row r="440" ht="14.25" customHeight="1"/>
-    <row r="441" ht="14.25" customHeight="1"/>
-    <row r="442" ht="14.25" customHeight="1"/>
-    <row r="443" ht="14.25" customHeight="1"/>
-    <row r="444" ht="14.25" customHeight="1"/>
-    <row r="445" ht="14.25" customHeight="1"/>
-    <row r="446" ht="14.25" customHeight="1"/>
-    <row r="447" ht="14.25" customHeight="1"/>
-    <row r="448" ht="14.25" customHeight="1"/>
-    <row r="449" ht="14.25" customHeight="1"/>
-    <row r="450" ht="14.25" customHeight="1"/>
-    <row r="451" ht="14.25" customHeight="1"/>
-    <row r="452" ht="14.25" customHeight="1"/>
-    <row r="453" ht="14.25" customHeight="1"/>
-    <row r="454" ht="14.25" customHeight="1"/>
-    <row r="455" ht="14.25" customHeight="1"/>
-    <row r="456" ht="14.25" customHeight="1"/>
-    <row r="457" ht="14.25" customHeight="1"/>
-    <row r="458" ht="14.25" customHeight="1"/>
-    <row r="459" ht="14.25" customHeight="1"/>
-    <row r="460" ht="14.25" customHeight="1"/>
-    <row r="461" ht="14.25" customHeight="1"/>
-    <row r="462" ht="14.25" customHeight="1"/>
-    <row r="463" ht="14.25" customHeight="1"/>
-    <row r="464" ht="14.25" customHeight="1"/>
-    <row r="465" ht="14.25" customHeight="1"/>
-    <row r="466" ht="14.25" customHeight="1"/>
-    <row r="467" ht="14.25" customHeight="1"/>
-    <row r="468" ht="14.25" customHeight="1"/>
-    <row r="469" ht="14.25" customHeight="1"/>
-    <row r="470" ht="14.25" customHeight="1"/>
-    <row r="471" ht="14.25" customHeight="1"/>
-    <row r="472" ht="14.25" customHeight="1"/>
-    <row r="473" ht="14.25" customHeight="1"/>
-    <row r="474" ht="14.25" customHeight="1"/>
-    <row r="475" ht="14.25" customHeight="1"/>
-    <row r="476" ht="14.25" customHeight="1"/>
-    <row r="477" ht="14.25" customHeight="1"/>
-    <row r="478" ht="14.25" customHeight="1"/>
-    <row r="479" ht="14.25" customHeight="1"/>
-    <row r="480" ht="14.25" customHeight="1"/>
-    <row r="481" ht="14.25" customHeight="1"/>
-    <row r="482" ht="14.25" customHeight="1"/>
-    <row r="483" ht="14.25" customHeight="1"/>
-    <row r="484" ht="14.25" customHeight="1"/>
-    <row r="485" ht="14.25" customHeight="1"/>
-    <row r="486" ht="14.25" customHeight="1"/>
-    <row r="487" ht="14.25" customHeight="1"/>
-    <row r="488" ht="14.25" customHeight="1"/>
-    <row r="489" ht="14.25" customHeight="1"/>
-    <row r="490" ht="14.25" customHeight="1"/>
-    <row r="491" ht="14.25" customHeight="1"/>
-    <row r="492" ht="14.25" customHeight="1"/>
-    <row r="493" ht="14.25" customHeight="1"/>
-    <row r="494" ht="14.25" customHeight="1"/>
-    <row r="495" ht="14.25" customHeight="1"/>
-    <row r="496" ht="14.25" customHeight="1"/>
-    <row r="497" ht="14.25" customHeight="1"/>
-    <row r="498" ht="14.25" customHeight="1"/>
-    <row r="499" ht="14.25" customHeight="1"/>
-    <row r="500" ht="14.25" customHeight="1"/>
-    <row r="501" ht="14.25" customHeight="1"/>
-    <row r="502" ht="14.25" customHeight="1"/>
-    <row r="503" ht="14.25" customHeight="1"/>
-    <row r="504" ht="14.25" customHeight="1"/>
-    <row r="505" ht="14.25" customHeight="1"/>
-    <row r="506" ht="14.25" customHeight="1"/>
-    <row r="507" ht="14.25" customHeight="1"/>
-    <row r="508" ht="14.25" customHeight="1"/>
-    <row r="509" ht="14.25" customHeight="1"/>
-    <row r="510" ht="14.25" customHeight="1"/>
-    <row r="511" ht="14.25" customHeight="1"/>
-    <row r="512" ht="14.25" customHeight="1"/>
-    <row r="513" ht="14.25" customHeight="1"/>
-    <row r="514" ht="14.25" customHeight="1"/>
-    <row r="515" ht="14.25" customHeight="1"/>
-    <row r="516" ht="14.25" customHeight="1"/>
-    <row r="517" ht="14.25" customHeight="1"/>
-    <row r="518" ht="14.25" customHeight="1"/>
-    <row r="519" ht="14.25" customHeight="1"/>
-    <row r="520" ht="14.25" customHeight="1"/>
-    <row r="521" ht="14.25" customHeight="1"/>
-    <row r="522" ht="14.25" customHeight="1"/>
-    <row r="523" ht="14.25" customHeight="1"/>
-    <row r="524" ht="14.25" customHeight="1"/>
-    <row r="525" ht="14.25" customHeight="1"/>
-    <row r="526" ht="14.25" customHeight="1"/>
-    <row r="527" ht="14.25" customHeight="1"/>
-    <row r="528" ht="14.25" customHeight="1"/>
-    <row r="529" ht="14.25" customHeight="1"/>
-    <row r="530" ht="14.25" customHeight="1"/>
-    <row r="531" ht="14.25" customHeight="1"/>
-    <row r="532" ht="14.25" customHeight="1"/>
-    <row r="533" ht="14.25" customHeight="1"/>
-    <row r="534" ht="14.25" customHeight="1"/>
-    <row r="535" ht="14.25" customHeight="1"/>
-    <row r="536" ht="14.25" customHeight="1"/>
-    <row r="537" ht="14.25" customHeight="1"/>
-    <row r="538" ht="14.25" customHeight="1"/>
-    <row r="539" ht="14.25" customHeight="1"/>
-    <row r="540" ht="14.25" customHeight="1"/>
-    <row r="541" ht="14.25" customHeight="1"/>
-    <row r="542" ht="14.25" customHeight="1"/>
-    <row r="543" ht="14.25" customHeight="1"/>
-    <row r="544" ht="14.25" customHeight="1"/>
-    <row r="545" ht="14.25" customHeight="1"/>
-    <row r="546" ht="14.25" customHeight="1"/>
-    <row r="547" ht="14.25" customHeight="1"/>
-    <row r="548" ht="14.25" customHeight="1"/>
-    <row r="549" ht="14.25" customHeight="1"/>
-    <row r="550" ht="14.25" customHeight="1"/>
-    <row r="551" ht="14.25" customHeight="1"/>
-    <row r="552" ht="14.25" customHeight="1"/>
-    <row r="553" ht="14.25" customHeight="1"/>
-    <row r="554" ht="14.25" customHeight="1"/>
-    <row r="555" ht="14.25" customHeight="1"/>
-    <row r="556" ht="14.25" customHeight="1"/>
-    <row r="557" ht="14.25" customHeight="1"/>
-    <row r="558" ht="14.25" customHeight="1"/>
-    <row r="559" ht="14.25" customHeight="1"/>
-    <row r="560" ht="14.25" customHeight="1"/>
-    <row r="561" ht="14.25" customHeight="1"/>
-    <row r="562" ht="14.25" customHeight="1"/>
-    <row r="563" ht="14.25" customHeight="1"/>
-    <row r="564" ht="14.25" customHeight="1"/>
-    <row r="565" ht="14.25" customHeight="1"/>
-    <row r="566" ht="14.25" customHeight="1"/>
-    <row r="567" ht="14.25" customHeight="1"/>
-    <row r="568" ht="14.25" customHeight="1"/>
-    <row r="569" ht="14.25" customHeight="1"/>
-    <row r="570" ht="14.25" customHeight="1"/>
-    <row r="571" ht="14.25" customHeight="1"/>
-    <row r="572" ht="14.25" customHeight="1"/>
-    <row r="573" ht="14.25" customHeight="1"/>
-    <row r="574" ht="14.25" customHeight="1"/>
-    <row r="575" ht="14.25" customHeight="1"/>
-    <row r="576" ht="14.25" customHeight="1"/>
-    <row r="577" ht="14.25" customHeight="1"/>
-    <row r="578" ht="14.25" customHeight="1"/>
-    <row r="579" ht="14.25" customHeight="1"/>
-    <row r="580" ht="14.25" customHeight="1"/>
-    <row r="581" ht="14.25" customHeight="1"/>
-    <row r="582" ht="14.25" customHeight="1"/>
-    <row r="583" ht="14.25" customHeight="1"/>
-    <row r="584" ht="14.25" customHeight="1"/>
-    <row r="585" ht="14.25" customHeight="1"/>
-    <row r="586" ht="14.25" customHeight="1"/>
-    <row r="587" ht="14.25" customHeight="1"/>
-    <row r="588" ht="14.25" customHeight="1"/>
-    <row r="589" ht="14.25" customHeight="1"/>
-    <row r="590" ht="14.25" customHeight="1"/>
-    <row r="591" ht="14.25" customHeight="1"/>
-    <row r="592" ht="14.25" customHeight="1"/>
-    <row r="593" ht="14.25" customHeight="1"/>
-    <row r="594" ht="14.25" customHeight="1"/>
-    <row r="595" ht="14.25" customHeight="1"/>
-    <row r="596" ht="14.25" customHeight="1"/>
-    <row r="597" ht="14.25" customHeight="1"/>
-    <row r="598" ht="14.25" customHeight="1"/>
-    <row r="599" ht="14.25" customHeight="1"/>
-    <row r="600" ht="14.25" customHeight="1"/>
-    <row r="601" ht="14.25" customHeight="1"/>
-    <row r="602" ht="14.25" customHeight="1"/>
-    <row r="603" ht="14.25" customHeight="1"/>
-    <row r="604" ht="14.25" customHeight="1"/>
-    <row r="605" ht="14.25" customHeight="1"/>
-    <row r="606" ht="14.25" customHeight="1"/>
-    <row r="607" ht="14.25" customHeight="1"/>
-    <row r="608" ht="14.25" customHeight="1"/>
-    <row r="609" ht="14.25" customHeight="1"/>
-    <row r="610" ht="14.25" customHeight="1"/>
-    <row r="611" ht="14.25" customHeight="1"/>
-    <row r="612" ht="14.25" customHeight="1"/>
-    <row r="613" ht="14.25" customHeight="1"/>
-    <row r="614" ht="14.25" customHeight="1"/>
-    <row r="615" ht="14.25" customHeight="1"/>
-    <row r="616" ht="14.25" customHeight="1"/>
-    <row r="617" ht="14.25" customHeight="1"/>
-    <row r="618" ht="14.25" customHeight="1"/>
-    <row r="619" ht="14.25" customHeight="1"/>
-    <row r="620" ht="14.25" customHeight="1"/>
-    <row r="621" ht="14.25" customHeight="1"/>
-    <row r="622" ht="14.25" customHeight="1"/>
-    <row r="623" ht="14.25" customHeight="1"/>
-    <row r="624" ht="14.25" customHeight="1"/>
-    <row r="625" ht="14.25" customHeight="1"/>
-    <row r="626" ht="14.25" customHeight="1"/>
-    <row r="627" ht="14.25" customHeight="1"/>
-    <row r="628" ht="14.25" customHeight="1"/>
-    <row r="629" ht="14.25" customHeight="1"/>
-    <row r="630" ht="14.25" customHeight="1"/>
-    <row r="631" ht="14.25" customHeight="1"/>
-    <row r="632" ht="14.25" customHeight="1"/>
-    <row r="633" ht="14.25" customHeight="1"/>
-    <row r="634" ht="14.25" customHeight="1"/>
-    <row r="635" ht="14.25" customHeight="1"/>
-    <row r="636" ht="14.25" customHeight="1"/>
-    <row r="637" ht="14.25" customHeight="1"/>
-    <row r="638" ht="14.25" customHeight="1"/>
-    <row r="639" ht="14.25" customHeight="1"/>
-    <row r="640" ht="14.25" customHeight="1"/>
-    <row r="641" ht="14.25" customHeight="1"/>
-    <row r="642" ht="14.25" customHeight="1"/>
-    <row r="643" ht="14.25" customHeight="1"/>
-    <row r="644" ht="14.25" customHeight="1"/>
-    <row r="645" ht="14.25" customHeight="1"/>
-    <row r="646" ht="14.25" customHeight="1"/>
-    <row r="647" ht="14.25" customHeight="1"/>
-    <row r="648" ht="14.25" customHeight="1"/>
-    <row r="649" ht="14.25" customHeight="1"/>
-    <row r="650" ht="14.25" customHeight="1"/>
-    <row r="651" ht="14.25" customHeight="1"/>
-    <row r="652" ht="14.25" customHeight="1"/>
-    <row r="653" ht="14.25" customHeight="1"/>
-    <row r="654" ht="14.25" customHeight="1"/>
-    <row r="655" ht="14.25" customHeight="1"/>
-    <row r="656" ht="14.25" customHeight="1"/>
-    <row r="657" ht="14.25" customHeight="1"/>
-    <row r="658" ht="14.25" customHeight="1"/>
-    <row r="659" ht="14.25" customHeight="1"/>
-    <row r="660" ht="14.25" customHeight="1"/>
-    <row r="661" ht="14.25" customHeight="1"/>
-    <row r="662" ht="14.25" customHeight="1"/>
-    <row r="663" ht="14.25" customHeight="1"/>
-    <row r="664" ht="14.25" customHeight="1"/>
-    <row r="665" ht="14.25" customHeight="1"/>
-    <row r="666" ht="14.25" customHeight="1"/>
-    <row r="667" ht="14.25" customHeight="1"/>
-    <row r="668" ht="14.25" customHeight="1"/>
-    <row r="669" ht="14.25" customHeight="1"/>
-    <row r="670" ht="14.25" customHeight="1"/>
-    <row r="671" ht="14.25" customHeight="1"/>
-    <row r="672" ht="14.25" customHeight="1"/>
-    <row r="673" ht="14.25" customHeight="1"/>
-    <row r="674" ht="14.25" customHeight="1"/>
-    <row r="675" ht="14.25" customHeight="1"/>
-    <row r="676" ht="14.25" customHeight="1"/>
-    <row r="677" ht="14.25" customHeight="1"/>
-    <row r="678" ht="14.25" customHeight="1"/>
-    <row r="679" ht="14.25" customHeight="1"/>
-    <row r="680" ht="14.25" customHeight="1"/>
-    <row r="681" ht="14.25" customHeight="1"/>
-    <row r="682" ht="14.25" customHeight="1"/>
-    <row r="683" ht="14.25" customHeight="1"/>
-    <row r="684" ht="14.25" customHeight="1"/>
-    <row r="685" ht="14.25" customHeight="1"/>
-    <row r="686" ht="14.25" customHeight="1"/>
-    <row r="687" ht="14.25" customHeight="1"/>
-    <row r="688" ht="14.25" customHeight="1"/>
-    <row r="689" ht="14.25" customHeight="1"/>
-    <row r="690" ht="14.25" customHeight="1"/>
-    <row r="691" ht="14.25" customHeight="1"/>
-    <row r="692" ht="14.25" customHeight="1"/>
-    <row r="693" ht="14.25" customHeight="1"/>
-    <row r="694" ht="14.25" customHeight="1"/>
-    <row r="695" ht="14.25" customHeight="1"/>
-    <row r="696" ht="14.25" customHeight="1"/>
-    <row r="697" ht="14.25" customHeight="1"/>
-    <row r="698" ht="14.25" customHeight="1"/>
-    <row r="699" ht="14.25" customHeight="1"/>
-    <row r="700" ht="14.25" customHeight="1"/>
-    <row r="701" ht="14.25" customHeight="1"/>
-    <row r="702" ht="14.25" customHeight="1"/>
-    <row r="703" ht="14.25" customHeight="1"/>
-    <row r="704" ht="14.25" customHeight="1"/>
-    <row r="705" ht="14.25" customHeight="1"/>
-    <row r="706" ht="14.25" customHeight="1"/>
-    <row r="707" ht="14.25" customHeight="1"/>
-    <row r="708" ht="14.25" customHeight="1"/>
-    <row r="709" ht="14.25" customHeight="1"/>
-    <row r="710" ht="14.25" customHeight="1"/>
-    <row r="711" ht="14.25" customHeight="1"/>
-    <row r="712" ht="14.25" customHeight="1"/>
-    <row r="713" ht="14.25" customHeight="1"/>
-    <row r="714" ht="14.25" customHeight="1"/>
-    <row r="715" ht="14.25" customHeight="1"/>
-    <row r="716" ht="14.25" customHeight="1"/>
-    <row r="717" ht="14.25" customHeight="1"/>
-    <row r="718" ht="14.25" customHeight="1"/>
-    <row r="719" ht="14.25" customHeight="1"/>
-    <row r="720" ht="14.25" customHeight="1"/>
-    <row r="721" ht="14.25" customHeight="1"/>
-    <row r="722" ht="14.25" customHeight="1"/>
-    <row r="723" ht="14.25" customHeight="1"/>
-    <row r="724" ht="14.25" customHeight="1"/>
-    <row r="725" ht="14.25" customHeight="1"/>
-    <row r="726" ht="14.25" customHeight="1"/>
-    <row r="727" ht="14.25" customHeight="1"/>
-    <row r="728" ht="14.25" customHeight="1"/>
-    <row r="729" ht="14.25" customHeight="1"/>
-    <row r="730" ht="14.25" customHeight="1"/>
-    <row r="731" ht="14.25" customHeight="1"/>
-    <row r="732" ht="14.25" customHeight="1"/>
-    <row r="733" ht="14.25" customHeight="1"/>
-    <row r="734" ht="14.25" customHeight="1"/>
-    <row r="735" ht="14.25" customHeight="1"/>
-    <row r="736" ht="14.25" customHeight="1"/>
-    <row r="737" ht="14.25" customHeight="1"/>
-    <row r="738" ht="14.25" customHeight="1"/>
-    <row r="739" ht="14.25" customHeight="1"/>
-    <row r="740" ht="14.25" customHeight="1"/>
-    <row r="741" ht="14.25" customHeight="1"/>
-    <row r="742" ht="14.25" customHeight="1"/>
-    <row r="743" ht="14.25" customHeight="1"/>
-    <row r="744" ht="14.25" customHeight="1"/>
-    <row r="745" ht="14.25" customHeight="1"/>
-    <row r="746" ht="14.25" customHeight="1"/>
-    <row r="747" ht="14.25" customHeight="1"/>
-    <row r="748" ht="14.25" customHeight="1"/>
-    <row r="749" ht="14.25" customHeight="1"/>
-    <row r="750" ht="14.25" customHeight="1"/>
-    <row r="751" ht="14.25" customHeight="1"/>
-    <row r="752" ht="14.25" customHeight="1"/>
-    <row r="753" ht="14.25" customHeight="1"/>
-    <row r="754" ht="14.25" customHeight="1"/>
-    <row r="755" ht="14.25" customHeight="1"/>
-    <row r="756" ht="14.25" customHeight="1"/>
-    <row r="757" ht="14.25" customHeight="1"/>
-    <row r="758" ht="14.25" customHeight="1"/>
-    <row r="759" ht="14.25" customHeight="1"/>
-    <row r="760" ht="14.25" customHeight="1"/>
-    <row r="761" ht="14.25" customHeight="1"/>
-    <row r="762" ht="14.25" customHeight="1"/>
-    <row r="763" ht="14.25" customHeight="1"/>
-    <row r="764" ht="14.25" customHeight="1"/>
-    <row r="765" ht="14.25" customHeight="1"/>
-    <row r="766" ht="14.25" customHeight="1"/>
-    <row r="767" ht="14.25" customHeight="1"/>
-    <row r="768" ht="14.25" customHeight="1"/>
-    <row r="769" ht="14.25" customHeight="1"/>
-    <row r="770" ht="14.25" customHeight="1"/>
-    <row r="771" ht="14.25" customHeight="1"/>
-    <row r="772" ht="14.25" customHeight="1"/>
-    <row r="773" ht="14.25" customHeight="1"/>
-    <row r="774" ht="14.25" customHeight="1"/>
-    <row r="775" ht="14.25" customHeight="1"/>
-    <row r="776" ht="14.25" customHeight="1"/>
-    <row r="777" ht="14.25" customHeight="1"/>
-    <row r="778" ht="14.25" customHeight="1"/>
-    <row r="779" ht="14.25" customHeight="1"/>
-    <row r="780" ht="14.25" customHeight="1"/>
-    <row r="781" ht="14.25" customHeight="1"/>
-    <row r="782" ht="14.25" customHeight="1"/>
-    <row r="783" ht="14.25" customHeight="1"/>
-    <row r="784" ht="14.25" customHeight="1"/>
-    <row r="785" ht="14.25" customHeight="1"/>
-    <row r="786" ht="14.25" customHeight="1"/>
-    <row r="787" ht="14.25" customHeight="1"/>
-    <row r="788" ht="14.25" customHeight="1"/>
-    <row r="789" ht="14.25" customHeight="1"/>
-    <row r="790" ht="14.25" customHeight="1"/>
-    <row r="791" ht="14.25" customHeight="1"/>
-    <row r="792" ht="14.25" customHeight="1"/>
-    <row r="793" ht="14.25" customHeight="1"/>
-    <row r="794" ht="14.25" customHeight="1"/>
-    <row r="795" ht="14.25" customHeight="1"/>
-    <row r="796" ht="14.25" customHeight="1"/>
-    <row r="797" ht="14.25" customHeight="1"/>
-    <row r="798" ht="14.25" customHeight="1"/>
-    <row r="799" ht="14.25" customHeight="1"/>
-    <row r="800" ht="14.25" customHeight="1"/>
-    <row r="801" ht="14.25" customHeight="1"/>
-    <row r="802" ht="14.25" customHeight="1"/>
-    <row r="803" ht="14.25" customHeight="1"/>
-    <row r="804" ht="14.25" customHeight="1"/>
-    <row r="805" ht="14.25" customHeight="1"/>
-    <row r="806" ht="14.25" customHeight="1"/>
-    <row r="807" ht="14.25" customHeight="1"/>
-    <row r="808" ht="14.25" customHeight="1"/>
-    <row r="809" ht="14.25" customHeight="1"/>
-    <row r="810" ht="14.25" customHeight="1"/>
-    <row r="811" ht="14.25" customHeight="1"/>
-    <row r="812" ht="14.25" customHeight="1"/>
-    <row r="813" ht="14.25" customHeight="1"/>
-    <row r="814" ht="14.25" customHeight="1"/>
-    <row r="815" ht="14.25" customHeight="1"/>
-    <row r="816" ht="14.25" customHeight="1"/>
-    <row r="817" ht="14.25" customHeight="1"/>
-    <row r="818" ht="14.25" customHeight="1"/>
-    <row r="819" ht="14.25" customHeight="1"/>
-    <row r="820" ht="14.25" customHeight="1"/>
-    <row r="821" ht="14.25" customHeight="1"/>
-    <row r="822" ht="14.25" customHeight="1"/>
-    <row r="823" ht="14.25" customHeight="1"/>
-    <row r="824" ht="14.25" customHeight="1"/>
-    <row r="825" ht="14.25" customHeight="1"/>
-    <row r="826" ht="14.25" customHeight="1"/>
-    <row r="827" ht="14.25" customHeight="1"/>
-    <row r="828" ht="14.25" customHeight="1"/>
-    <row r="829" ht="14.25" customHeight="1"/>
-    <row r="830" ht="14.25" customHeight="1"/>
-    <row r="831" ht="14.25" customHeight="1"/>
-    <row r="832" ht="14.25" customHeight="1"/>
-    <row r="833" ht="14.25" customHeight="1"/>
-    <row r="834" ht="14.25" customHeight="1"/>
-    <row r="835" ht="14.25" customHeight="1"/>
-    <row r="836" ht="14.25" customHeight="1"/>
-    <row r="837" ht="14.25" customHeight="1"/>
-    <row r="838" ht="14.25" customHeight="1"/>
-    <row r="839" ht="14.25" customHeight="1"/>
-    <row r="840" ht="14.25" customHeight="1"/>
-    <row r="841" ht="14.25" customHeight="1"/>
-    <row r="842" ht="14.25" customHeight="1"/>
-    <row r="843" ht="14.25" customHeight="1"/>
-    <row r="844" ht="14.25" customHeight="1"/>
-    <row r="845" ht="14.25" customHeight="1"/>
-    <row r="846" ht="14.25" customHeight="1"/>
-    <row r="847" ht="14.25" customHeight="1"/>
-    <row r="848" ht="14.25" customHeight="1"/>
-    <row r="849" ht="14.25" customHeight="1"/>
-    <row r="850" ht="14.25" customHeight="1"/>
-    <row r="851" ht="14.25" customHeight="1"/>
-    <row r="852" ht="14.25" customHeight="1"/>
-    <row r="853" ht="14.25" customHeight="1"/>
-    <row r="854" ht="14.25" customHeight="1"/>
-    <row r="855" ht="14.25" customHeight="1"/>
-    <row r="856" ht="14.25" customHeight="1"/>
-    <row r="857" ht="14.25" customHeight="1"/>
-    <row r="858" ht="14.25" customHeight="1"/>
-    <row r="859" ht="14.25" customHeight="1"/>
-    <row r="860" ht="14.25" customHeight="1"/>
-    <row r="861" ht="14.25" customHeight="1"/>
-    <row r="862" ht="14.25" customHeight="1"/>
-    <row r="863" ht="14.25" customHeight="1"/>
-    <row r="864" ht="14.25" customHeight="1"/>
-    <row r="865" ht="14.25" customHeight="1"/>
-    <row r="866" ht="14.25" customHeight="1"/>
-    <row r="867" ht="14.25" customHeight="1"/>
-    <row r="868" ht="14.25" customHeight="1"/>
-    <row r="869" ht="14.25" customHeight="1"/>
-    <row r="870" ht="14.25" customHeight="1"/>
-    <row r="871" ht="14.25" customHeight="1"/>
-    <row r="872" ht="14.25" customHeight="1"/>
-    <row r="873" ht="14.25" customHeight="1"/>
-    <row r="874" ht="14.25" customHeight="1"/>
-    <row r="875" ht="14.25" customHeight="1"/>
-    <row r="876" ht="14.25" customHeight="1"/>
-    <row r="877" ht="14.25" customHeight="1"/>
-    <row r="878" ht="14.25" customHeight="1"/>
-    <row r="879" ht="14.25" customHeight="1"/>
-    <row r="880" ht="14.25" customHeight="1"/>
-    <row r="881" ht="14.25" customHeight="1"/>
-    <row r="882" ht="14.25" customHeight="1"/>
-    <row r="883" ht="14.25" customHeight="1"/>
-    <row r="884" ht="14.25" customHeight="1"/>
-    <row r="885" ht="14.25" customHeight="1"/>
-    <row r="886" ht="14.25" customHeight="1"/>
-    <row r="887" ht="14.25" customHeight="1"/>
-    <row r="888" ht="14.25" customHeight="1"/>
-    <row r="889" ht="14.25" customHeight="1"/>
-    <row r="890" ht="14.25" customHeight="1"/>
-    <row r="891" ht="14.25" customHeight="1"/>
-    <row r="892" ht="14.25" customHeight="1"/>
-    <row r="893" ht="14.25" customHeight="1"/>
-    <row r="894" ht="14.25" customHeight="1"/>
-    <row r="895" ht="14.25" customHeight="1"/>
-    <row r="896" ht="14.25" customHeight="1"/>
-    <row r="897" ht="14.25" customHeight="1"/>
-    <row r="898" ht="14.25" customHeight="1"/>
-    <row r="899" ht="14.25" customHeight="1"/>
-    <row r="900" ht="14.25" customHeight="1"/>
-    <row r="901" ht="14.25" customHeight="1"/>
-    <row r="902" ht="14.25" customHeight="1"/>
-    <row r="903" ht="14.25" customHeight="1"/>
-    <row r="904" ht="14.25" customHeight="1"/>
-    <row r="905" ht="14.25" customHeight="1"/>
-    <row r="906" ht="14.25" customHeight="1"/>
-    <row r="907" ht="14.25" customHeight="1"/>
-    <row r="908" ht="14.25" customHeight="1"/>
-    <row r="909" ht="14.25" customHeight="1"/>
-    <row r="910" ht="14.25" customHeight="1"/>
-    <row r="911" ht="14.25" customHeight="1"/>
-    <row r="912" ht="14.25" customHeight="1"/>
-    <row r="913" ht="14.25" customHeight="1"/>
-    <row r="914" ht="14.25" customHeight="1"/>
-    <row r="915" ht="14.25" customHeight="1"/>
-    <row r="916" ht="14.25" customHeight="1"/>
-    <row r="917" ht="14.25" customHeight="1"/>
-    <row r="918" ht="14.25" customHeight="1"/>
-    <row r="919" ht="14.25" customHeight="1"/>
-    <row r="920" ht="14.25" customHeight="1"/>
-    <row r="921" ht="14.25" customHeight="1"/>
-    <row r="922" ht="14.25" customHeight="1"/>
-    <row r="923" ht="14.25" customHeight="1"/>
-    <row r="924" ht="14.25" customHeight="1"/>
-    <row r="925" ht="14.25" customHeight="1"/>
-    <row r="926" ht="14.25" customHeight="1"/>
-    <row r="927" ht="14.25" customHeight="1"/>
-    <row r="928" ht="14.25" customHeight="1"/>
-    <row r="929" ht="14.25" customHeight="1"/>
-    <row r="930" ht="14.25" customHeight="1"/>
-    <row r="931" ht="14.25" customHeight="1"/>
-    <row r="932" ht="14.25" customHeight="1"/>
-    <row r="933" ht="14.25" customHeight="1"/>
-    <row r="934" ht="14.25" customHeight="1"/>
-    <row r="935" ht="14.25" customHeight="1"/>
-    <row r="936" ht="14.25" customHeight="1"/>
-    <row r="937" ht="14.25" customHeight="1"/>
-    <row r="938" ht="14.25" customHeight="1"/>
-    <row r="939" ht="14.25" customHeight="1"/>
-    <row r="940" ht="14.25" customHeight="1"/>
-    <row r="941" ht="14.25" customHeight="1"/>
-    <row r="942" ht="14.25" customHeight="1"/>
-    <row r="943" ht="14.25" customHeight="1"/>
-    <row r="944" ht="14.25" customHeight="1"/>
-    <row r="945" ht="14.25" customHeight="1"/>
-    <row r="946" ht="14.25" customHeight="1"/>
-    <row r="947" ht="14.25" customHeight="1"/>
-    <row r="948" ht="14.25" customHeight="1"/>
-    <row r="949" ht="14.25" customHeight="1"/>
-    <row r="950" ht="14.25" customHeight="1"/>
-    <row r="951" ht="14.25" customHeight="1"/>
-    <row r="952" ht="14.25" customHeight="1"/>
-    <row r="953" ht="14.25" customHeight="1"/>
-    <row r="954" ht="14.25" customHeight="1"/>
-    <row r="955" ht="14.25" customHeight="1"/>
-    <row r="956" ht="14.25" customHeight="1"/>
-    <row r="957" ht="14.25" customHeight="1"/>
-    <row r="958" ht="14.25" customHeight="1"/>
-    <row r="959" ht="14.25" customHeight="1"/>
-    <row r="960" ht="14.25" customHeight="1"/>
-    <row r="961" ht="14.25" customHeight="1"/>
-    <row r="962" ht="14.25" customHeight="1"/>
-    <row r="963" ht="14.25" customHeight="1"/>
-    <row r="964" ht="14.25" customHeight="1"/>
-    <row r="965" ht="14.25" customHeight="1"/>
-    <row r="966" ht="14.25" customHeight="1"/>
-    <row r="967" ht="14.25" customHeight="1"/>
-    <row r="968" ht="14.25" customHeight="1"/>
-    <row r="969" ht="14.25" customHeight="1"/>
-    <row r="970" ht="14.25" customHeight="1"/>
-    <row r="971" ht="14.25" customHeight="1"/>
-    <row r="972" ht="14.25" customHeight="1"/>
-    <row r="973" ht="14.25" customHeight="1"/>
-    <row r="974" ht="14.25" customHeight="1"/>
-    <row r="975" ht="14.25" customHeight="1"/>
-    <row r="976" ht="14.25" customHeight="1"/>
-    <row r="977" ht="14.25" customHeight="1"/>
-    <row r="978" ht="14.25" customHeight="1"/>
-    <row r="979" ht="14.25" customHeight="1"/>
-    <row r="980" ht="14.25" customHeight="1"/>
-    <row r="981" ht="14.25" customHeight="1"/>
-    <row r="982" ht="14.25" customHeight="1"/>
-    <row r="983" ht="14.25" customHeight="1"/>
-    <row r="984" ht="14.25" customHeight="1"/>
-    <row r="985" ht="14.25" customHeight="1"/>
-    <row r="986" ht="14.25" customHeight="1"/>
-    <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
-    <row r="989" ht="14.25" customHeight="1"/>
-    <row r="990" ht="14.25" customHeight="1"/>
-    <row r="991" ht="14.25" customHeight="1"/>
-    <row r="992" ht="14.25" customHeight="1"/>
-    <row r="993" ht="14.25" customHeight="1"/>
-    <row r="994" ht="14.25" customHeight="1"/>
-    <row r="995" ht="14.25" customHeight="1"/>
-    <row r="996" ht="14.25" customHeight="1"/>
-    <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
-    <row r="1001" ht="14.25" customHeight="1"/>
-    <row r="1002" ht="14.25" customHeight="1"/>
-    <row r="1003" ht="14.25" customHeight="1"/>
-    <row r="1004" ht="14.25" customHeight="1"/>
-    <row r="1005" ht="14.25" customHeight="1"/>
-    <row r="1006" ht="14.25" customHeight="1"/>
-    <row r="1007" ht="14.25" customHeight="1"/>
-    <row r="1008" ht="14.25" customHeight="1"/>
-    <row r="1009" ht="14.25" customHeight="1"/>
-    <row r="1010" ht="14.25" customHeight="1"/>
-    <row r="1011" ht="14.25" customHeight="1"/>
-    <row r="1012" ht="14.25" customHeight="1"/>
-    <row r="1013" ht="14.25" customHeight="1"/>
-    <row r="1014" ht="14.25" customHeight="1"/>
-    <row r="1015" ht="14.25" customHeight="1"/>
-    <row r="1016" ht="14.25" customHeight="1"/>
-    <row r="1017" ht="14.25" customHeight="1"/>
-    <row r="1018" ht="14.25" customHeight="1"/>
-    <row r="1019" ht="14.25" customHeight="1"/>
-    <row r="1020" ht="14.25" customHeight="1"/>
-    <row r="1021" ht="14.25" customHeight="1"/>
-    <row r="1022" ht="14.25" customHeight="1"/>
-    <row r="1023" ht="14.25" customHeight="1"/>
-    <row r="1024" ht="14.25" customHeight="1"/>
-    <row r="1025" ht="14.25" customHeight="1"/>
-    <row r="1026" ht="14.25" customHeight="1"/>
-    <row r="1027" ht="14.25" customHeight="1"/>
-    <row r="1028" ht="14.25" customHeight="1"/>
-    <row r="1029" ht="14.25" customHeight="1"/>
-    <row r="1030" ht="14.25" customHeight="1"/>
-    <row r="1031" ht="14.25" customHeight="1"/>
-    <row r="1032" ht="14.25" customHeight="1"/>
-    <row r="1033" ht="14.25" customHeight="1"/>
-    <row r="1034" ht="14.25" customHeight="1"/>
-    <row r="1035" ht="14.25" customHeight="1"/>
-    <row r="1036" ht="14.25" customHeight="1"/>
-    <row r="1037" ht="14.25" customHeight="1"/>
-    <row r="1038" ht="14.25" customHeight="1"/>
-    <row r="1039" ht="14.25" customHeight="1"/>
-    <row r="1040" ht="14.25" customHeight="1"/>
-    <row r="1041" ht="14.25" customHeight="1"/>
-    <row r="1042" ht="14.25" customHeight="1"/>
-    <row r="1043" ht="14.25" customHeight="1"/>
-    <row r="1044" ht="14.25" customHeight="1"/>
-    <row r="1045" ht="14.25" customHeight="1"/>
-    <row r="1046" ht="14.25" customHeight="1"/>
-    <row r="1047" ht="14.25" customHeight="1"/>
-    <row r="1048" ht="14.25" customHeight="1"/>
-    <row r="1049" ht="14.25" customHeight="1"/>
-    <row r="1050" ht="14.25" customHeight="1"/>
-    <row r="1051" ht="14.25" customHeight="1"/>
-    <row r="1052" ht="14.25" customHeight="1"/>
-    <row r="1053" ht="14.25" customHeight="1"/>
-    <row r="1054" ht="14.25" customHeight="1"/>
-    <row r="1055" ht="14.25" customHeight="1"/>
-    <row r="1056" ht="14.25" customHeight="1"/>
-    <row r="1057" ht="14.25" customHeight="1"/>
-    <row r="1058" ht="14.25" customHeight="1"/>
-    <row r="1059" ht="14.25" customHeight="1"/>
-    <row r="1060" ht="14.25" customHeight="1"/>
-    <row r="1061" ht="14.25" customHeight="1"/>
-    <row r="1062" ht="14.25" customHeight="1"/>
-    <row r="1063" ht="14.25" customHeight="1"/>
-    <row r="1064" ht="14.25" customHeight="1"/>
-    <row r="1065" ht="14.25" customHeight="1"/>
-    <row r="1066" ht="14.25" customHeight="1"/>
-    <row r="1067" ht="14.25" customHeight="1"/>
-    <row r="1068" ht="14.25" customHeight="1"/>
-    <row r="1069" ht="14.25" customHeight="1"/>
-    <row r="1070" ht="14.25" customHeight="1"/>
-    <row r="1071" ht="14.25" customHeight="1"/>
-    <row r="1072" ht="14.25" customHeight="1"/>
-    <row r="1073" ht="14.25" customHeight="1"/>
-    <row r="1074" ht="14.25" customHeight="1"/>
-    <row r="1075" ht="14.25" customHeight="1"/>
-    <row r="1076" ht="14.25" customHeight="1"/>
-    <row r="1077" ht="14.25" customHeight="1"/>
-    <row r="1078" ht="14.25" customHeight="1"/>
-    <row r="1079" ht="14.25" customHeight="1"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>